<commit_message>
Update ETF pipeline outputs and project docs
</commit_message>
<xml_diff>
--- a/providers/xtrackers/2026-07-05/xtrackers_etf_export.xlsx
+++ b/providers/xtrackers/2026-07-05/xtrackers_etf_export.xlsx
@@ -24975,449 +24975,449 @@
     <x:mergeCell ref="B446:R446"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink ref="B8:B8" r:id="R20ff195ded1042f8" display="https://etf.dws.com//en-gb/IE00002ZKAP0-europe-equity-enhanced-active-ucits-etf-1c/"/>
-    <x:hyperlink ref="B9:B9" r:id="R6c10af6ec96245af" display="https://etf.dws.com//en-gb/IE00004DJ199-msci-world-swap-ii-ucits-etf-1d/"/>
-    <x:hyperlink ref="B10:B10" r:id="Rf428ac303dce4e11" display="https://etf.dws.com//en-gb/IE0000K7HU41-msci-usa-information-technology-ucits-etf-1c/"/>
-    <x:hyperlink ref="B11:B11" r:id="R19459b814cc942a6" display="https://etf.dws.com//en-gb/IE0000MMQ5M5-msci-usa-esg-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B12:B12" r:id="Raef6d4f9ef044e53" display="https://etf.dws.com//en-gb/IE0001JH5CB4-europe-net-zero-pathway-paris-aligned-ucits-etf-1c/"/>
-    <x:hyperlink ref="B13:B13" r:id="R69b209617a93494c" display="https://etf.dws.com//en-gb/IE0001TLQX55-s-p-500-garp-ucits-etf-1c/"/>
-    <x:hyperlink ref="B14:B14" r:id="R146fd7aa70594497" display="https://etf.dws.com//en-gb/IE00028H9QJ8-usd-corporate-green-bond-ucits-etf-1c-eur-hedged/"/>
-    <x:hyperlink ref="B15:B15" r:id="R6b84d94e6a4b4f21" display="https://etf.dws.com//en-gb/IE0002EI5AG0-s-p-500-equal-weight-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B16:B16" r:id="Rb9b4833b303e4670" display="https://etf.dws.com//en-gb/IE0002GFATQ6-s-p-500-equal-weight-ucits-etf-3c-chf-hedged/"/>
-    <x:hyperlink ref="B17:B17" r:id="R9adb7f67ad8a4560" display="https://etf.dws.com//en-gb/IE0002PGSLZ5-us-equity-enhanced-active-ucits-etf-1c/"/>
-    <x:hyperlink ref="B18:B18" r:id="R87eb796d7bce47f9" display="https://etf.dws.com//en-gb/IE0002ZM3JI1-usa-net-zero-pathway-paris-aligned-ucits-etf-1c/"/>
-    <x:hyperlink ref="B19:B19" r:id="R51cd7f956cb34ff6" display="https://etf.dws.com//en-gb/IE00036F4K40-msci-global-sdg-3-good-health-ucits-etf-1c/"/>
-    <x:hyperlink ref="B20:B20" r:id="Rda633f232711436a" display="https://etf.dws.com//en-gb/IE0003NQ0IY5-msci-world-quality-esg-ucits-etf-1c/"/>
-    <x:hyperlink ref="B21:B21" r:id="Re6f5604c531e49b6" display="https://etf.dws.com//en-gb/IE0003W9O921-usd-corporate-green-bond-ucits-etf-2c/"/>
-    <x:hyperlink ref="B22:B22" r:id="R3ec671574a91408b" display="https://etf.dws.com//en-gb/IE000472H9T4-nasdaq-100-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B23:B23" r:id="R844e4172c94a404d" display="https://etf.dws.com//en-gb/IE0004KLW911-esg-usd-emerging-markets-bond-quality-weighted-ucits-etf-1c/"/>
-    <x:hyperlink ref="B24:B24" r:id="Ra0437d4c42194145" display="https://etf.dws.com//en-gb/IE0004MFRED4-s-p-500-equal-weight-scored-screened-ucits-etf-1c/"/>
-    <x:hyperlink ref="B25:B25" r:id="R6622fdff12134862" display="https://etf.dws.com//en-gb/IE0004ZJGWT9-msci-europe-esg-ucits-etf-1d/"/>
-    <x:hyperlink ref="B26:B26" r:id="Rb1944c406ee24f55" display="https://etf.dws.com//en-gb/IE0005E47AH7-msci-global-sdg-9-industry-innovation-infrastructure-ucits-etf-1c/"/>
-    <x:hyperlink ref="B27:B27" r:id="R2830494314504d5f" display="https://etf.dws.com//en-gb/IE0006FDYJF8-msci-japan-climate-transition-ucits-etf-1d/"/>
-    <x:hyperlink ref="B28:B28" r:id="Raf360f68e0874a04" display="https://etf.dws.com//en-gb/IE0006FFX5U1-msci-innovation-ucits-etf-1c/"/>
-    <x:hyperlink ref="B29:B29" r:id="Rac7f14af72354bfa" display="https://etf.dws.com//en-gb/IE0006GNB732-eur-high-yield-corporate-bond-sri-pab-ucits-etf-1c/"/>
-    <x:hyperlink ref="B30:B30" r:id="R7bb04a1f8d984820" display="https://etf.dws.com//en-gb/IE0006I3NZF8-msci-usa-consumer-discretionary-ucits-etf-1c/"/>
-    <x:hyperlink ref="B31:B31" r:id="Rc4e264fde919470e" display="https://etf.dws.com//en-gb/IE0006WW1TQ4-msci-world-ex-usa-ucits-etf-1c/"/>
-    <x:hyperlink ref="B32:B32" r:id="Rd6df65c64e7a40d6" display="https://etf.dws.com//en-gb/IE0006YM7D84-usd-high-yield-corporate-bond-screened-ucits-etf-1c/"/>
-    <x:hyperlink ref="B33:B33" r:id="Rf44b34f3bdc64d05" display="https://etf.dws.com//en-gb/IE00074JLU02-japan-net-zero-pathway-paris-aligned-ucits-etf-1c/"/>
-    <x:hyperlink ref="B34:B34" r:id="Rf5651f299a004bba" display="https://etf.dws.com//en-gb/IE0007ULOZS8-s-p-500-scored-screened-ucits-etf-1c/"/>
-    <x:hyperlink ref="B35:B35" r:id="Rdd3937a7e691476f" display="https://etf.dws.com//en-gb/IE0007WJ6B10-msci-global-clean-water-sanitation-ucits-etf-1c/"/>
-    <x:hyperlink ref="B36:B36" r:id="R455dcf09ddff4470" display="https://etf.dws.com//en-gb/IE0008YN0OY8-msci-world-minimum-volatility-esg-ucits-etf-1c/"/>
-    <x:hyperlink ref="B37:B37" r:id="Rddfca06ee2c24a67" display="https://etf.dws.com//en-gb/IE00094GSCQ4-world-equity-enhanced-active-ucits-etf-1c/"/>
-    <x:hyperlink ref="B38:B38" r:id="R80196fb5c3ec4454" display="https://etf.dws.com//en-gb/IE0009KLWT21-msci-world-ucits-etf-3c-chf-hedged/"/>
-    <x:hyperlink ref="B39:B39" r:id="Rbbb5be1bc0c2497c" display="https://etf.dws.com//en-gb/IE000BO2Y0T8-msci-nordic-ucits-etf-1c/"/>
-    <x:hyperlink ref="B40:B40" r:id="R544f839d68ab4632" display="https://etf.dws.com//en-gb/IE000CXLGK86-s-p-500-equal-weight-ucits-etf-2d/"/>
-    <x:hyperlink ref="B41:B41" r:id="Rc12e2c63ad2a4a6e" display="https://etf.dws.com//en-gb/IE000DNSAS54-msci-emerging-markets-climate-transition-ucits-etf-1c/"/>
-    <x:hyperlink ref="B42:B42" r:id="R6e883e97d2934b55" display="https://etf.dws.com//en-gb/IE000DVHJV46-s-p-500-market-leaders-ucits-etf-1c/"/>
-    <x:hyperlink ref="B43:B43" r:id="Rb7836f1b52914a9c" display="https://etf.dws.com//en-gb/IE000E0V65D8-world-biodiversity-focus-sri-ucits-etf-1c/"/>
-    <x:hyperlink ref="B44:B44" r:id="Rfabb2162c3ce4589" display="https://etf.dws.com//en-gb/IE000E4BATC9-msci-world-esg-ucits-etf-1d/"/>
-    <x:hyperlink ref="B45:B45" r:id="Rba085743812e4b9a" display="https://etf.dws.com//en-gb/IE000ER61U30-msci-europe-small-cap-esg-ucits-etf-1c/"/>
-    <x:hyperlink ref="B46:B46" r:id="R8a200acd6dbf4ad5" display="https://etf.dws.com//en-gb/IE000EVOVOG1-msci-usa-positioning-screened-ucits-etf-1d/"/>
-    <x:hyperlink ref="B47:B47" r:id="R879b4347a5c04325" display="https://etf.dws.com//en-gb/IE000EXUE0G2-nasdaq-100-swap-ucits-etf-1d/"/>
-    <x:hyperlink ref="B48:B48" r:id="R493ac2806ad3483c" display="https://etf.dws.com//en-gb/IE000F04HGE5-floating-rate-notes-active-ucits-etf-1c/"/>
-    <x:hyperlink ref="B49:B49" r:id="Rdec005258791483f" display="https://etf.dws.com//en-gb/IE000F354Q61-msci-world-small-cap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B50:B50" r:id="R56c96438f6ab4168" display="https://etf.dws.com//en-gb/IE000FL46JJ1-s-p-500-equal-weight-swap-ucits-etf-1d/"/>
-    <x:hyperlink ref="B51:B51" r:id="R0e2d4cd68f904c71" display="https://etf.dws.com//en-gb/IE000FO05UG4-s-p-500-swap-ii-ucits-etf-1d/"/>
-    <x:hyperlink ref="B52:B52" r:id="R2783fb7ca04246b9" display="https://etf.dws.com//en-gb/IE000FO1A5D1-s-p-500-equal-weight-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B53:B53" r:id="R614c19efacc84db7" display="https://etf.dws.com//en-gb/IE000FW16TX1-msci-usa-swap-ii-ucits-etf-1d/"/>
-    <x:hyperlink ref="B54:B54" r:id="R790791b7c2c8468a" display="https://etf.dws.com//en-gb/IE000GF6QTP6-s-p-500-equal-weight-scored-screened-ucits-etf-3c-chf-hedged/"/>
-    <x:hyperlink ref="B55:B55" r:id="Rb21d4e22b53e471d" display="https://etf.dws.com//en-gb/IE000GWA2J58-msci-emerging-markets-ucits-etf-1d/"/>
-    <x:hyperlink ref="B56:B56" r:id="Rcdee8cfe00304f14" display="https://etf.dws.com//en-gb/IE000GYDNJS5-msci-usa-climate-transition-ucits-etf-1d/"/>
-    <x:hyperlink ref="B57:B57" r:id="Rb99cc574eb5246c5" display="https://etf.dws.com//en-gb/IE000HT7E0B1-nordic-net-zero-pathway-paris-aligned-ucits-etf-1c/"/>
-    <x:hyperlink ref="B58:B58" r:id="R855b19b47b204ba2" display="https://etf.dws.com//en-gb/IE000HY30YW6-s-p-500-swap-ii-ucits-etf-1c/"/>
-    <x:hyperlink ref="B59:B59" r:id="R2e68fad4263743ec" display="https://etf.dws.com//en-gb/IE000IDLWOL4-s-p-500-equal-weight-scored-screened-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B60:B60" r:id="Rba0dc31f33d44bdc" display="https://etf.dws.com//en-gb/IE000INYW0A7-msci-world-swap-ii-ucits-etf-1c/"/>
-    <x:hyperlink ref="B61:B61" r:id="Rcc6eee2f03bb463c" display="https://etf.dws.com//en-gb/IE000ISS8DB2-msci-world-small-cap-ucits-etf-1d/"/>
-    <x:hyperlink ref="B62:B62" r:id="R5875ab96bb22408d" display="https://etf.dws.com//en-gb/IE000JZYIUN0-msci-global-sdg-7-affordable-and-clean-energy-ucits-etf-1c/"/>
-    <x:hyperlink ref="B63:B63" r:id="Rc983bb2222374bee" display="https://etf.dws.com//en-gb/IE000KD0BZ68-msci-genomic-healthcare-innovation-ucits-etf-1c/"/>
-    <x:hyperlink ref="B64:B64" r:id="Re6401e6b6094498e" display="https://etf.dws.com//en-gb/IE000L2IS494-msci-global-social-fairness-contributors-ucits-etf-1c/"/>
-    <x:hyperlink ref="B65:B65" r:id="Redbe786e92834e6c" display="https://etf.dws.com//en-gb/IE000L6ZMMC4-ftse-all-world-ucits-etf-1c/"/>
-    <x:hyperlink ref="B66:B66" r:id="Rb03594c8fb67440c" display="https://etf.dws.com//en-gb/IE000LAUZQT6-msci-world-value-esg-ucits-etf-1c/"/>
-    <x:hyperlink ref="B67:B67" r:id="R5256ad87491d4f43" display="https://etf.dws.com//en-gb/IE000LOSV2D0-usa-biodiversity-focus-sri-ucits-etf-1c/"/>
-    <x:hyperlink ref="B68:B68" r:id="R5a804db75373425b" display="https://etf.dws.com//en-gb/IE000M8F3JA6-global-growth-leaders-active-ucits-etf-1c/"/>
-    <x:hyperlink ref="B69:B69" r:id="Rda9fce7e8346472b" display="https://etf.dws.com//en-gb/IE000MCVFK47-eur-corporate-green-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B70:B70" r:id="R902b5b4384d74098" display="https://etf.dws.com//en-gb/IE000ME8PWJ4-msci-world-utilities-ucits-etf-1d/"/>
-    <x:hyperlink ref="B71:B71" r:id="Rf351b4bd2cda4408" display="https://etf.dws.com//en-gb/IE000MF9SZ46-msci-nordic-ucits-etf-2c-gbp-hedged/"/>
-    <x:hyperlink ref="B72:B72" r:id="R196ba58a886e4031" display="https://etf.dws.com//en-gb/IE000N5GJDD7-s-p-500-equal-weight-ucits-etf-1d-gbp-hedged/"/>
-    <x:hyperlink ref="B73:B73" r:id="R8898acd2a7f74e47" display="https://etf.dws.com//en-gb/IE000N9MLVT1-msci-europe-climate-transition-ucits-etf-1c/"/>
-    <x:hyperlink ref="B74:B74" r:id="Rdfeb35f826fd4ce3" display="https://etf.dws.com//en-gb/IE000NS5HRY9-msci-world-high-dividend-yield-esg-ucits-etf-1d/"/>
-    <x:hyperlink ref="B75:B75" r:id="Rda4ecc40dc3d4ae2" display="https://etf.dws.com//en-gb/IE000O7Q2E56-electrification-technologies-smart-grid-ucits-etf-1c/"/>
-    <x:hyperlink ref="B76:B76" r:id="Re92ad260562d484e" display="https://etf.dws.com//en-gb/IE000ONQ3X90-msci-world-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B77:B77" r:id="R5544ae8243464cc4" display="https://etf.dws.com//en-gb/IE000P4AYI47-msci-world-climate-transition-ucits-etf-1c/"/>
-    <x:hyperlink ref="B78:B78" r:id="R26f9dc1eb2674c3d" display="https://etf.dws.com//en-gb/IE000PDUVTF3-msci-usa-swap-ii-ucits-etf-1c/"/>
-    <x:hyperlink ref="B79:B79" r:id="Rf0f1044aaca04934" display="https://etf.dws.com//en-gb/IE000PSF3A70-msci-global-sdgs-ucits-etf-1c/"/>
-    <x:hyperlink ref="B80:B80" r:id="R2a5464ed7be34a7b" display="https://etf.dws.com//en-gb/IE000QVYFUT7-india-government-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B81:B81" r:id="R3c2629c4bf454919" display="https://etf.dws.com//en-gb/IE000RNHIKK1-msci-usa-health-care-ucits-etf-1c/"/>
-    <x:hyperlink ref="B82:B82" r:id="R875e5f2966f74be8" display="https://etf.dws.com//en-gb/IE000SRQBBT6-s-p-500-defensive-shareholder-yield-ucits-etf-1c/"/>
-    <x:hyperlink ref="B83:B83" r:id="R576ec75f4798434c" display="https://etf.dws.com//en-gb/IE000SZ25OI0-s-p-500-equal-weight-scored-screened-ucits-etf-4c-gbp-hedged/"/>
-    <x:hyperlink ref="B84:B84" r:id="Rca6de01f93944db9" display="https://etf.dws.com//en-gb/IE000TL3PL69-msci-world-momentum-esg-ucits-etf-1c/"/>
-    <x:hyperlink ref="B85:B85" r:id="R66b5c56f758341ad" display="https://etf.dws.com//en-gb/IE000TSML5I8-msci-usa-screened-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B86:B86" r:id="R7d5f13ceea2249f9" display="https://etf.dws.com//en-gb/IE000TZT8TI0-emerging-markets-net-zero-pathway-paris-aligned-ucits-etf-1c/"/>
-    <x:hyperlink ref="B87:B87" r:id="Ra8b8763e1b834e30" display="https://etf.dws.com//en-gb/IE000UATQPE2-msci-world-small-cap-esg-ucits-etf-1c/"/>
-    <x:hyperlink ref="B88:B88" r:id="R6ab13d5c99ed4ff0" display="https://etf.dws.com//en-gb/IE000UMV0L21-msci-usa-esg-ucits-etf-1d/"/>
-    <x:hyperlink ref="B89:B89" r:id="Rd48d845d83624fd8" display="https://etf.dws.com//en-gb/IE000UP2BIZ9-s-p-500-ucits-etf-4d/"/>
-    <x:hyperlink ref="B90:B90" r:id="R2acbf36c53a1473e" display="https://etf.dws.com//en-gb/IE000UX5WPU4-iboxx-eur-corporate-bond-yield-plus-ucits-etf-1c/"/>
-    <x:hyperlink ref="B91:B91" r:id="R0faff32afefd4113" display="https://etf.dws.com//en-gb/IE000UZCJS58-world-net-zero-pathway-paris-aligned-ucits-etf-1c/"/>
-    <x:hyperlink ref="B92:B92" r:id="R43c8e15ef17f4e6e" display="https://etf.dws.com//en-gb/IE000V04SL39-msci-usa-high-dividend-yield-esg-ucits-etf-1d/"/>
-    <x:hyperlink ref="B93:B93" r:id="R370bb3286b594a5a" display="https://etf.dws.com//en-gb/IE000V0GDVU7-msci-global-sdg-11-sustainable-cities-ucits-etf-1c/"/>
-    <x:hyperlink ref="B94:B94" r:id="Rdcc1b5c2e261436b" display="https://etf.dws.com//en-gb/IE000VCBWFL8-msci-emu-high-dividend-yield-esg-ucits-etf-1d/"/>
-    <x:hyperlink ref="B95:B95" r:id="R5ec15b5d801b497d" display="https://etf.dws.com//en-gb/IE000VCTBRW6-msci-world-industrials-ucits-etf-1d/"/>
-    <x:hyperlink ref="B96:B96" r:id="Rd16a0d31a770413e" display="https://etf.dws.com//en-gb/IE000VXC51U5-msci-ac-world-screened-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B97:B97" r:id="Rea5e5db89749458a" display="https://etf.dws.com//en-gb/IE000W6L2AI3-msci-emu-climate-transition-ucits-etf-1c/"/>
-    <x:hyperlink ref="B98:B98" r:id="R30f5d5e932e3404e" display="https://etf.dws.com//en-gb/IE000WGF1X01-msci-ac-world-screened-ucits-etf-5c-usd-hedged/"/>
-    <x:hyperlink ref="B99:B99" r:id="R7545e0f4e137474d" display="https://etf.dws.com//en-gb/IE000WHO5BF2-usd-high-yield-corporate-bond-screened-ucits-etf-2c-gbp-hedged/"/>
-    <x:hyperlink ref="B100:B100" r:id="Rab495e6393b5477b" display="https://etf.dws.com//en-gb/IE000WQ16XQ4-msci-europe-high-dividend-yield-esg-ucits-etf-1d/"/>
-    <x:hyperlink ref="B101:B101" r:id="R4f0d13951d894d89" display="https://etf.dws.com//en-gb/IE000X1GW0A7-msci-world-imi-ucits-etf-1c/"/>
-    <x:hyperlink ref="B102:B102" r:id="R02d76914cd8c4f33" display="https://etf.dws.com//en-gb/IE000X4A4GV2-global-equity-top-active-ucits-etf-1c/"/>
-    <x:hyperlink ref="B103:B103" r:id="R9e05acf61a564ee8" display="https://etf.dws.com//en-gb/IE000X5MRP46-msci-usa-financials-ucits-etf-1c/"/>
-    <x:hyperlink ref="B104:B104" r:id="R22326f4066d34ee0" display="https://etf.dws.com//en-gb/IE000X63FXN4-usd-corporate-green-bond-ucits-etf-1d-gbp-hedged/"/>
-    <x:hyperlink ref="B105:B105" r:id="R390df6f6d55e40ba" display="https://etf.dws.com//en-gb/IE000X6Z71P5-msci-usa-consumer-staples-ucits-etf-1c/"/>
-    <x:hyperlink ref="B106:B106" r:id="R606e6ffe769e4343" display="https://etf.dws.com//en-gb/IE000XOQ9TK4-msci-next-generation-internet-innovation-ucits-etf-1c/"/>
-    <x:hyperlink ref="B107:B107" r:id="R76dec0339f3e45cf" display="https://etf.dws.com//en-gb/IE000Y6L6LE6-emu-net-zero-pathway-paris-aligned-ucits-etf-1c/"/>
-    <x:hyperlink ref="B108:B108" r:id="R1d285655fffb4429" display="https://etf.dws.com//en-gb/IE000Y6ZXZ48-msci-global-circular-economy-ucits-etf-1c/"/>
-    <x:hyperlink ref="B109:B109" r:id="R22bdfbb6cc464633" display="https://etf.dws.com//en-gb/IE000YDOORK7-msci-fintech-innovation-ucits-etf-1c/"/>
-    <x:hyperlink ref="B110:B110" r:id="R4b4b1a26d2c14ecc" display="https://etf.dws.com//en-gb/IE000YKHGYN2-ftse-all-world-ex-us-ucits-etf-1c/"/>
-    <x:hyperlink ref="B111:B111" r:id="Rdad6abc494524ed1" display="https://etf.dws.com//en-gb/IE000Z0FC0G5-msci-world-ex-usa-ucits-etf-1d/"/>
-    <x:hyperlink ref="B112:B112" r:id="R134dd1249dea46a1" display="https://etf.dws.com//en-gb/IE000Z9SJA06-s-p-500-ucits-etf-4c/"/>
-    <x:hyperlink ref="B113:B113" r:id="R87a221b7cbed47d5" display="https://etf.dws.com//en-gb/IE00B3Y8D011-portfolio-income-ucits-etf-1d/"/>
-    <x:hyperlink ref="B114:B114" r:id="Rdf247c96d37f4f31" display="https://etf.dws.com//en-gb/IE00B8KMSQ34-s-p-500-ucits-etf-3c-chf-hedged/"/>
-    <x:hyperlink ref="B115:B115" r:id="Raceb3be4c616425d" display="https://etf.dws.com//en-gb/IE00B9MRHC27-msci-nordic-ucits-etf-1d/"/>
-    <x:hyperlink ref="B116:B116" r:id="Ra529a15e1df6426f" display="https://etf.dws.com//en-gb/IE00B9MRJJ36-mdax-esg-screened-ucits-etf-1d/"/>
-    <x:hyperlink ref="B117:B117" r:id="R09cab07280774f83" display="https://etf.dws.com//en-gb/IE00BCHWNQ94-msci-world-screened-ucits-etf-1d/"/>
-    <x:hyperlink ref="B118:B118" r:id="R206dd58c9d564fc8" display="https://etf.dws.com//en-gb/IE00BCHWNS19-msci-usa-energy-ucits-etf-1d/"/>
-    <x:hyperlink ref="B119:B119" r:id="R8bd2d9e6c2d54d70" display="https://etf.dws.com//en-gb/IE00BCHWNT26-msci-usa-financials-ucits-etf-1d/"/>
-    <x:hyperlink ref="B120:B120" r:id="R030de45411ae4e54" display="https://etf.dws.com//en-gb/IE00BCHWNV48-msci-usa-industrials-ucits-etf-1d/"/>
-    <x:hyperlink ref="B121:B121" r:id="R3d20e70e98434b4c" display="https://etf.dws.com//en-gb/IE00BCHWNW54-msci-usa-health-care-ucits-etf-1d/"/>
-    <x:hyperlink ref="B122:B122" r:id="R20b54589f9e74448" display="https://etf.dws.com//en-gb/IE00BD4DX952-esg-usd-emerging-markets-bond-quality-weighted-ucits-etf-1d/"/>
-    <x:hyperlink ref="B123:B123" r:id="Rf9ae6d137cd644e3" display="https://etf.dws.com//en-gb/IE00BD4DXB77-esg-usd-emerging-markets-bond-quality-weighted-ucits-etf-2d-eur-hedged/"/>
-    <x:hyperlink ref="B124:B124" r:id="Rf42126d1edbb45c6" display="https://etf.dws.com//en-gb/IE00BDB7J586-msci-usa-minimum-volatility-ucits-etf-1d/"/>
-    <x:hyperlink ref="B125:B125" r:id="Rda86413423344973" display="https://etf.dws.com//en-gb/IE00BDGN9Z19-msci-emu-screened-ucits-etf-1d/"/>
-    <x:hyperlink ref="B126:B126" r:id="R90e9b7dce47240a7" display="https://etf.dws.com//en-gb/IE00BDR5HM97-usd-high-yield-corporate-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B127:B127" r:id="R01b41601c0344f18" display="https://etf.dws.com//en-gb/IE00BDR5HN05-usd-high-yield-corporate-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B128:B128" r:id="Re8c0d76ca4064cce" display="https://etf.dws.com//en-gb/IE00BDVPTJ63-msci-usa-banks-ucits-etf-1d/"/>
-    <x:hyperlink ref="B129:B129" r:id="R0b10881bec3d4bab" display="https://etf.dws.com//en-gb/IE00BF8J5974-usd-corporate-bond-short-duration-sri-pab-ucits-etf-1d/"/>
-    <x:hyperlink ref="B130:B130" r:id="R239f252f94854161" display="https://etf.dws.com//en-gb/IE00BFMKQ930-usd-corporate-bond-short-duration-sri-pab-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B131:B131" r:id="R2f3597d62dd74118" display="https://etf.dws.com//en-gb/IE00BFMKQC67-usd-corporate-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B132:B132" r:id="R3f5c3a8daed042a1" display="https://etf.dws.com//en-gb/IE00BFMNHK08-msci-europe-esg-ucits-etf-1c/"/>
-    <x:hyperlink ref="B133:B133" r:id="Rf1afcfdbf616439b" display="https://etf.dws.com//en-gb/IE00BFMNPS42-msci-usa-esg-ucits-etf-1c/"/>
-    <x:hyperlink ref="B134:B134" r:id="Rb56e376c4e754c0a" display="https://etf.dws.com//en-gb/IE00BG04LT92-usd-high-yield-corporate-bond-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B135:B135" r:id="Rb4a9d6dec4af4a18" display="https://etf.dws.com//en-gb/IE00BG04LV15-usd-high-yield-corporate-bond-ucits-etf-4d-gbp-hedged/"/>
-    <x:hyperlink ref="B136:B136" r:id="R3aec9b39a3cb4930" display="https://etf.dws.com//en-gb/IE00BG04LY46-usd-corporate-bond-ucits-etf-5d-gbp-hedged/"/>
-    <x:hyperlink ref="B137:B137" r:id="Rec8599ac68514824" display="https://etf.dws.com//en-gb/IE00BG04LZ52-msci-usa-ucits-etf-3c-chf-hedged/"/>
-    <x:hyperlink ref="B138:B138" r:id="R48d4e1020ea74324" display="https://etf.dws.com//en-gb/IE00BG04M077-msci-usa-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B139:B139" r:id="R20fe7b90adfd4f4e" display="https://etf.dws.com//en-gb/IE00BG36TC12-msci-japan-esg-ucits-etf-1c/"/>
-    <x:hyperlink ref="B140:B140" r:id="R18b88d3c95ac41eb" display="https://etf.dws.com//en-gb/IE00BG370F43-msci-emerging-markets-esg-ucits-etf-1c/"/>
-    <x:hyperlink ref="B141:B141" r:id="R92b390069cb645ac" display="https://etf.dws.com//en-gb/IE00BGHQ0G80-msci-ac-world-screened-ucits-etf-1c/"/>
-    <x:hyperlink ref="B142:B142" r:id="Rf71e349426e4453e" display="https://etf.dws.com//en-gb/IE00BGJWX091-s-p-500-ucits-etf-1d-eur-hedged/"/>
-    <x:hyperlink ref="B143:B143" r:id="Rac7625f4322f4261" display="https://etf.dws.com//en-gb/IE00BGQYRQ28-msci-usa-consumer-staples-ucits-etf-1d/"/>
-    <x:hyperlink ref="B144:B144" r:id="Re1513236963c4f59" display="https://etf.dws.com//en-gb/IE00BGQYRR35-msci-usa-consumer-discretionary-ucits-etf-1d/"/>
-    <x:hyperlink ref="B145:B145" r:id="Rbf3beadf2fcd406e" display="https://etf.dws.com//en-gb/IE00BGQYRS42-msci-usa-information-technology-ucits-etf-1d/"/>
-    <x:hyperlink ref="B146:B146" r:id="R3bc63d78b7494d41" display="https://etf.dws.com//en-gb/IE00BGV5VM45-s-p-europe-ex-uk-ucits-etf-1d/"/>
-    <x:hyperlink ref="B147:B147" r:id="R0f945416587d4763" display="https://etf.dws.com//en-gb/IE00BGV5VN51-artificial-intelligence-big-data-ucits-etf-1c/"/>
-    <x:hyperlink ref="B148:B148" r:id="Recb39580518e48d8" display="https://etf.dws.com//en-gb/IE00BGV5VR99-future-mobility-ucits-etf-1c/"/>
-    <x:hyperlink ref="B149:B149" r:id="R1a2b7a3194934676" display="https://etf.dws.com//en-gb/IE00BH361H73-msci-north-america-high-dividend-yield-ucits-etf-1c/"/>
-    <x:hyperlink ref="B150:B150" r:id="Rffce09eca3844cd8" display="https://etf.dws.com//en-gb/IE00BJ0KDQ92-msci-world-ucits-etf-1c/"/>
-    <x:hyperlink ref="B151:B151" r:id="R49418012fa314483" display="https://etf.dws.com//en-gb/IE00BJ0KDR00-msci-usa-ucits-etf-1c/"/>
-    <x:hyperlink ref="B152:B152" r:id="Rcd007b295f064a7f" display="https://etf.dws.com//en-gb/IE00BJZ2DC62-msci-usa-screened-ucits-etf-1c/"/>
-    <x:hyperlink ref="B153:B153" r:id="R24d8c2cde6014f90" display="https://etf.dws.com//en-gb/IE00BJZ2DD79-russell-2000-ucits-etf-1c/"/>
-    <x:hyperlink ref="B154:B154" r:id="R2acbd092e23f49e8" display="https://etf.dws.com//en-gb/IE00BK1PV445-msci-usa-ucits-etf-1d/"/>
-    <x:hyperlink ref="B155:B155" r:id="R03f89efe45ba43ec" display="https://etf.dws.com//en-gb/IE00BK1PV551-msci-world-ucits-etf-1d/"/>
-    <x:hyperlink ref="B156:B156" r:id="R12b2c846d3cc4a3f" display="https://etf.dws.com//en-gb/IE00BL25JL35-msci-world-quality-ucits-etf-1c/"/>
-    <x:hyperlink ref="B157:B157" r:id="Rcadb6aabda0f443b" display="https://etf.dws.com//en-gb/IE00BL25JM42-msci-world-value-ucits-etf-1c/"/>
-    <x:hyperlink ref="B158:B158" r:id="Rc75c929ca479447a" display="https://etf.dws.com//en-gb/IE00BL25JN58-msci-world-minimum-volatility-ucits-etf-1c/"/>
-    <x:hyperlink ref="B159:B159" r:id="Rd9c60001fdf94402" display="https://etf.dws.com//en-gb/IE00BL25JP72-msci-world-momentum-ucits-etf-1c/"/>
-    <x:hyperlink ref="B160:B160" r:id="R131436e07a904425" display="https://etf.dws.com//en-gb/IE00BL58LJ19-usd-corporate-bond-sri-pab-ucits-etf-1c/"/>
-    <x:hyperlink ref="B161:B161" r:id="Ra8c50f306fe04231" display="https://etf.dws.com//en-gb/IE00BL58LL31-usd-corporate-bond-sri-pab-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B162:B162" r:id="R897af697619e41aa" display="https://etf.dws.com//en-gb/IE00BLNMYC90-s-p-500-equal-weight-ucits-etf-1c/"/>
-    <x:hyperlink ref="B163:B163" r:id="R752ac9bd0a684275" display="https://etf.dws.com//en-gb/IE00BM67HJ62-msci-emerging-markets-ex-china-ucits-etf-1c/"/>
-    <x:hyperlink ref="B164:B164" r:id="Rc510037c6c9e4583" display="https://etf.dws.com//en-gb/IE00BM67HK77-msci-world-health-care-ucits-etf-1c/"/>
-    <x:hyperlink ref="B165:B165" r:id="R436f697b4315420d" display="https://etf.dws.com//en-gb/IE00BM67HL84-msci-world-financials-ucits-etf-1c/"/>
-    <x:hyperlink ref="B166:B166" r:id="Rdd7e9616edfa4f86" display="https://etf.dws.com//en-gb/IE00BM67HM91-msci-world-energy-ucits-etf-1c/"/>
-    <x:hyperlink ref="B167:B167" r:id="R9b8c651b2b524dbe" display="https://etf.dws.com//en-gb/IE00BM67HN09-msci-world-consumer-staples-ucits-etf-1c/"/>
-    <x:hyperlink ref="B168:B168" r:id="R687a297bc8c6436f" display="https://etf.dws.com//en-gb/IE00BM67HP23-msci-world-consumer-discretionary-ucits-etf-1c/"/>
-    <x:hyperlink ref="B169:B169" r:id="R00ad5b99d2d04371" display="https://etf.dws.com//en-gb/IE00BM67HQ30-msci-world-utilities-ucits-etf-1c/"/>
-    <x:hyperlink ref="B170:B170" r:id="R64353ef4c0d34729" display="https://etf.dws.com//en-gb/IE00BM67HR47-msci-world-communication-services-ucits-etf-1c/"/>
-    <x:hyperlink ref="B171:B171" r:id="R4332d342d57a497e" display="https://etf.dws.com//en-gb/IE00BM67HS53-msci-world-materials-ucits-etf-1c/"/>
-    <x:hyperlink ref="B172:B172" r:id="R6250aa62b3174ab8" display="https://etf.dws.com//en-gb/IE00BM67HT60-msci-world-information-technology-ucits-etf-1c/"/>
-    <x:hyperlink ref="B173:B173" r:id="Re1e493b832444f1d" display="https://etf.dws.com//en-gb/IE00BM67HV82-msci-world-industrials-ucits-etf-1c/"/>
-    <x:hyperlink ref="B174:B174" r:id="R1526723e99174605" display="https://etf.dws.com//en-gb/IE00BM67HW99-s-p-500-ucits-etf-1c-eur-hedged/"/>
-    <x:hyperlink ref="B175:B175" r:id="R7468f1dc5a384e30" display="https://etf.dws.com//en-gb/IE00BM67HX07-s-p-500-ucits-etf-2c-gbp-hedged/"/>
-    <x:hyperlink ref="B176:B176" r:id="R0f4d9983de7a444a" display="https://etf.dws.com//en-gb/IE00BM97MR69-us-treasuries-ultrashort-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B177:B177" r:id="Rb6d1542ce01142ea" display="https://etf.dws.com//en-gb/IE00BM97MV06-us-treasuries-ultrashort-bond-ucits-etf-3c-mxn-hedged/"/>
-    <x:hyperlink ref="B178:B178" r:id="R63d0311ad7b94752" display="https://etf.dws.com//en-gb/IE00BMCFJ320-usd-corporate-bond-ucits-etf-6c-mxn-hedged/"/>
-    <x:hyperlink ref="B179:B179" r:id="Re93436de0b0e43e3" display="https://etf.dws.com//en-gb/IE00BMFKG444-nasdaq-100-ucits-etf-1c/"/>
-    <x:hyperlink ref="B180:B180" r:id="Rfba012d719914ccd" display="https://etf.dws.com//en-gb/IE00BMY76136-msci-world-esg-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B181:B181" r:id="R880d7bc2dabd4e11" display="https://etf.dws.com//en-gb/IE00BN2BCY94-developed-green-real-estate-esg-ucits-etf-1c/"/>
-    <x:hyperlink ref="B182:B182" r:id="Rf87b848ed8a14829" display="https://etf.dws.com//en-gb/IE00BNC1G699-msci-emu-esg-ucits-etf-1c/"/>
-    <x:hyperlink ref="B183:B183" r:id="R70d9cd95bdef4e25" display="https://etf.dws.com//en-gb/IE00BNC1G707-msci-usa-communication-services-ucits-etf-1d/"/>
-    <x:hyperlink ref="B184:B184" r:id="Rdfc62f0ef84744da" display="https://etf.dws.com//en-gb/IE00BNKF6C99-stoxx-european-market-leaders-ucits-etf-1c/"/>
-    <x:hyperlink ref="B185:B185" r:id="R52e77264dcff44eb" display="https://etf.dws.com//en-gb/IE00BP8FKB21-ftse-developed-europe-ex-uk-real-estate-ucits-etf-1c/"/>
-    <x:hyperlink ref="B186:B186" r:id="R72fde5b969d245fa" display="https://etf.dws.com//en-gb/IE00BPVLQD13-msci-japan-screened-ucits-etf-1d/"/>
-    <x:hyperlink ref="B187:B187" r:id="Rcb69a3a703ad4672" display="https://etf.dws.com//en-gb/IE00BPVLQF37-msci-japan-screened-ucits-etf-2d-gbp-hedged/"/>
-    <x:hyperlink ref="B188:B188" r:id="R3f29a452540f4f18" display="https://etf.dws.com//en-gb/IE00BQXKVQ19-msci-gcc-select-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B189:B189" r:id="R5210937e38e24193" display="https://etf.dws.com//en-gb/IE00BRB36B93-msci-japan-screened-ucits-etf-3c-eur-hedged/"/>
-    <x:hyperlink ref="B190:B190" r:id="R1651ce6114b24456" display="https://etf.dws.com//en-gb/IE00BTGD1B38-msci-japan-screened-ucits-etf-4c-usd-hedged/"/>
-    <x:hyperlink ref="B191:B191" r:id="R652e0ed8e40542bb" display="https://etf.dws.com//en-gb/IE00BTJRMP35-msci-emerging-markets-ucits-etf-1c/"/>
-    <x:hyperlink ref="B192:B192" r:id="R0485efc1a27f4828" display="https://etf.dws.com//en-gb/IE00BYPHT736-iboxx-eur-corporate-bond-yield-plus-ucits-etf-1d/"/>
-    <x:hyperlink ref="B193:B193" r:id="R5e1aa762ef8a40dc" display="https://etf.dws.com//en-gb/IE00BYZNF849-global-infrastructure-esg-ucits-etf-1c/"/>
-    <x:hyperlink ref="B194:B194" r:id="R64c968caf258472d" display="https://etf.dws.com//en-gb/IE00BZ02LR44-msci-world-esg-ucits-etf-1c/"/>
-    <x:hyperlink ref="B195:B195" r:id="R20d3b8a4dfd24a0d" display="https://etf.dws.com//en-gb/IE00BZ036H21-usd-corporate-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B196:B196" r:id="Rbb2a7c27fce84da8" display="https://etf.dws.com//en-gb/IE00BZ036J45-usd-corporate-bond-ucits-etf-2d-eur-hedged/"/>
-    <x:hyperlink ref="B197:B197" r:id="Re2ecc7ef4af749d8" display="https://etf.dws.com//en-gb/IE00BZ1BS790-msci-world-ucits-etf-2d-gbp-hedged/"/>
-    <x:hyperlink ref="B198:B198" r:id="Ra2df0822e5eb44ef" display="https://etf.dws.com//en-gb/LU0274208692-msci-world-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B199:B199" r:id="R048d0abe251449bd" display="https://etf.dws.com//en-gb/LU0274209237-msci-europe-ucits-etf-1c/"/>
-    <x:hyperlink ref="B200:B200" r:id="R472d9b1c54804b58" display="https://etf.dws.com//en-gb/LU0274209740-msci-japan-ucits-etf-1c/"/>
-    <x:hyperlink ref="B201:B201" r:id="R7d53cf2976d64bc9" display="https://etf.dws.com//en-gb/LU0274210672-msci-usa-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B202:B202" r:id="Red56ca728c1d4e7c" display="https://etf.dws.com//en-gb/LU0274211217-euro-stoxx-50-ucits-etf-1d/"/>
-    <x:hyperlink ref="B203:B203" r:id="R3a0b423479c84119" display="https://etf.dws.com//en-gb/LU0274211480-dax-ucits-etf-1c/"/>
-    <x:hyperlink ref="B204:B204" r:id="R4d151b2a711544dd" display="https://etf.dws.com//en-gb/LU0274212538-ftse-mib-ucits-etf-1d/"/>
-    <x:hyperlink ref="B205:B205" r:id="Ra1b3f00bdf0c44ad" display="https://etf.dws.com//en-gb/LU0274221281-switzerland-ucits-etf-1d/"/>
-    <x:hyperlink ref="B206:B206" r:id="R876c8958220f4a20" display="https://etf.dws.com//en-gb/LU0290355717-eurozone-government-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B207:B207" r:id="R7e2268b148c94a56" display="https://etf.dws.com//en-gb/LU0290356871-eurozone-government-bond-1-3-ucits-etf-1c/"/>
-    <x:hyperlink ref="B208:B208" r:id="Rc40343b2fe0041f5" display="https://etf.dws.com//en-gb/LU0290356954-eurozone-government-bond-3-5-ucits-etf-1c/"/>
-    <x:hyperlink ref="B209:B209" r:id="R76bee3f88dbf41c7" display="https://etf.dws.com//en-gb/LU0290357176-eurozone-government-bond-5-7-ucits-etf-1c/"/>
-    <x:hyperlink ref="B210:B210" r:id="Red7c5a16a1ce49a6" display="https://etf.dws.com//en-gb/LU0290357259-eurozone-government-bond-7-10-ucits-etf-1c/"/>
-    <x:hyperlink ref="B211:B211" r:id="Rcbbcecb7eb8541c9" display="https://etf.dws.com//en-gb/LU0290357507-eurozone-government-bond-15-30-ucits-etf-1c/"/>
-    <x:hyperlink ref="B212:B212" r:id="R49e63fdddd6b40e6" display="https://etf.dws.com//en-gb/LU0290357846-eurozone-government-bond-25-ucits-etf-1c/"/>
-    <x:hyperlink ref="B213:B213" r:id="R044ae4c336314c69" display="https://etf.dws.com//en-gb/LU0290357929-global-inflation-linked-bond-ucits-etf-1c-eur-hedged/"/>
-    <x:hyperlink ref="B214:B214" r:id="R526af8ef280e410f" display="https://etf.dws.com//en-gb/LU0290358224-eurozone-inflation-linked-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B215:B215" r:id="Rfc74227ccd4c4f03" display="https://etf.dws.com//en-gb/LU0290358497-eur-overnight-rate-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B216:B216" r:id="R577bbe70eace46d5" display="https://etf.dws.com//en-gb/LU0292095535-euro-stoxx-quality-dividend-ucits-etf-1d/"/>
-    <x:hyperlink ref="B217:B217" r:id="R789a23a0b3f24242" display="https://etf.dws.com//en-gb/LU0292096186-stoxx-global-select-dividend-100-swap-ucits-etf-1d/"/>
-    <x:hyperlink ref="B218:B218" r:id="Rabc9a39ff8504ebc" display="https://etf.dws.com//en-gb/LU0292097234-ftse-100-income-ucits-etf-1d/"/>
-    <x:hyperlink ref="B219:B219" r:id="R498f0273d38e4ac2" display="https://etf.dws.com//en-gb/LU0292097317-ftse-250-ucits-etf-1d/"/>
-    <x:hyperlink ref="B220:B220" r:id="R8a2efabd43f14908" display="https://etf.dws.com//en-gb/LU0292097747-msci-uk-esg-ucits-etf-1d/"/>
-    <x:hyperlink ref="B221:B221" r:id="R010bfcef0f7142ce" display="https://etf.dws.com//en-gb/LU0292100046-msci-korea-ucits-etf-1c/"/>
-    <x:hyperlink ref="B222:B222" r:id="R53d732bc9911496d" display="https://etf.dws.com//en-gb/LU0292100806-msci-europe-materials-ucits-etf-1c/"/>
-    <x:hyperlink ref="B223:B223" r:id="Rd4ddd427b2784614" display="https://etf.dws.com//en-gb/LU0292103222-msci-europe-health-care-ucits-etf-1c/"/>
-    <x:hyperlink ref="B224:B224" r:id="R15ef47e746d5407e" display="https://etf.dws.com//en-gb/LU0292103651-msci-europe-financials-ucits-etf-1c/"/>
-    <x:hyperlink ref="B225:B225" r:id="R191b894539984ac3" display="https://etf.dws.com//en-gb/LU0292104030-msci-europe-communication-services-ucits-etf-1c/"/>
-    <x:hyperlink ref="B226:B226" r:id="R340ae1204da04c88" display="https://etf.dws.com//en-gb/LU0292104469-msci-europe-information-technology-ucits-etf-1c/"/>
-    <x:hyperlink ref="B227:B227" r:id="Rd2a088bded40494e" display="https://etf.dws.com//en-gb/LU0292104899-msci-europe-utilities-ucits-etf-1c/"/>
-    <x:hyperlink ref="B228:B228" r:id="R567d1b38374a40a7" display="https://etf.dws.com//en-gb/LU0292105359-msci-europe-consumer-staples-ucits-etf-1c/"/>
-    <x:hyperlink ref="B229:B229" r:id="R5babde79a7ad4e29" display="https://etf.dws.com//en-gb/LU0292106084-msci-europe-industrials-ucits-etf-1c/"/>
-    <x:hyperlink ref="B230:B230" r:id="R87482b38ec734769" display="https://etf.dws.com//en-gb/LU0292106167-bloomberg-commodity-ex-agriculture-livestock-swap-ucits-etf-1c-eur-hedged/"/>
-    <x:hyperlink ref="B231:B231" r:id="R3f1fe32c0baf4529" display="https://etf.dws.com//en-gb/LU0292106241-shortdax-daily-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B232:B232" r:id="R1ad3ed9b15054883" display="https://etf.dws.com//en-gb/LU0292106753-euro-stoxx-50-short-daily-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B233:B233" r:id="Rfbcb0cc3f7c04ca9" display="https://etf.dws.com//en-gb/LU0292107645-msci-emerging-markets-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B234:B234" r:id="Re321d0d944f94cc5" display="https://etf.dws.com//en-gb/LU0292107991-msci-em-asia-screened-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B235:B235" r:id="R939abeda82094435" display="https://etf.dws.com//en-gb/LU0292108619-msci-em-latin-america-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B236:B236" r:id="R3d0cd7b5ac1c4483" display="https://etf.dws.com//en-gb/LU0292109005-msci-em-europe-middle-east-africa-esg-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B237:B237" r:id="R035ad797a83a4938" display="https://etf.dws.com//en-gb/LU0292109187-msci-taiwan-ucits-etf-1c/"/>
-    <x:hyperlink ref="B238:B238" r:id="R5296c03f47314f24" display="https://etf.dws.com//en-gb/LU0292109344-msci-brazil-ucits-etf-1c/"/>
-    <x:hyperlink ref="B239:B239" r:id="R8cb2605576784e22" display="https://etf.dws.com//en-gb/LU0292109690-nifty-50-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B240:B240" r:id="R2ad827faa8ca4703" display="https://etf.dws.com//en-gb/LU0292109856-msci-china-a-ucits-etf-1c/"/>
-    <x:hyperlink ref="B241:B241" r:id="Re0182a9ad4b94c97" display="https://etf.dws.com//en-gb/LU0321462870-itraxx-crossover-short-daily-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B242:B242" r:id="Rb6988db43dd24471" display="https://etf.dws.com//en-gb/LU0321462953-j-p-morgan-usd-emerging-markets-bond-ucits-etf-1c-eur-hedged/"/>
-    <x:hyperlink ref="B243:B243" r:id="Rbbbf1ba595cc466b" display="https://etf.dws.com//en-gb/LU0321464652-gbp-overnight-rate-swap-ucits-etf-1d/"/>
-    <x:hyperlink ref="B244:B244" r:id="R66c94ae6d4794a68" display="https://etf.dws.com//en-gb/LU0321465469-usd-overnight-rate-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B245:B245" r:id="R6d300386d5e24162" display="https://etf.dws.com//en-gb/LU0322248146-sli-ucits-etf-1d/"/>
-    <x:hyperlink ref="B246:B246" r:id="Rcbd4b2a1788b4fb3" display="https://etf.dws.com//en-gb/LU0322250712-lpx-private-equity-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B247:B247" r:id="R5c01a2820dd44350" display="https://etf.dws.com//en-gb/LU0322250985-cac-40-ucits-etf-1d/"/>
-    <x:hyperlink ref="B248:B248" r:id="Rd7941128608f4d76" display="https://etf.dws.com//en-gb/LU0322251520-s-p-500-inverse-daily-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B249:B249" r:id="R3d98654723524380" display="https://etf.dws.com//en-gb/LU0322252171-msci-ac-asia-ex-japan-esg-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B250:B250" r:id="R002105cebac648e9" display="https://etf.dws.com//en-gb/LU0322252338-msci-pacific-ex-japan-ucits-etf-1c/"/>
-    <x:hyperlink ref="B251:B251" r:id="R4ae29e2f9f0c4582" display="https://etf.dws.com//en-gb/LU0322252924-vietnam-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B252:B252" r:id="R662227f3a0884678" display="https://etf.dws.com//en-gb/LU0322253229-s-p-global-infrastructure-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B253:B253" r:id="R3fec26ed028c4471" display="https://etf.dws.com//en-gb/LU0322253732-msci-europe-screened-ucits-etf-1c/"/>
-    <x:hyperlink ref="B254:B254" r:id="Rf110243fa27543c0" display="https://etf.dws.com//en-gb/LU0322253906-msci-europe-small-cap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B255:B255" r:id="R1e300997f6de40cd" display="https://etf.dws.com//en-gb/LU0328473581-ftse-100-short-daily-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B256:B256" r:id="Rcea50fa36d334bf6" display="https://etf.dws.com//en-gb/LU0328474803-s-p-asx-200-ucits-etf-1d/"/>
-    <x:hyperlink ref="B257:B257" r:id="R024e4af513954821" display="https://etf.dws.com//en-gb/LU0328475792-stoxx-europe-600-ucits-etf-1c/"/>
-    <x:hyperlink ref="B258:B258" r:id="Rc5d4a59af6ff4502" display="https://etf.dws.com//en-gb/LU0328476410-s-p-select-frontier-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B259:B259" r:id="R265abc48ee4b4918" display="https://etf.dws.com//en-gb/LU0335044896-eur-overnight-rate-swap-ucits-etf-1d/"/>
-    <x:hyperlink ref="B260:B260" r:id="Reef9d39435ca4fb4" display="https://etf.dws.com//en-gb/LU0378818131-global-government-bond-ucits-etf-1c-eur-hedged/"/>
-    <x:hyperlink ref="B261:B261" r:id="R2ef227cd88444529" display="https://etf.dws.com//en-gb/LU0378818560-singapore-government-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B262:B262" r:id="Rc2ce644d36bc4bd9" display="https://etf.dws.com//en-gb/LU0380865021-euro-stoxx-50-ucits-etf-1c/"/>
-    <x:hyperlink ref="B263:B263" r:id="R1188cb8848e746ee" display="https://etf.dws.com//en-gb/LU0397221945-portfolio-ucits-etf-1c/"/>
-    <x:hyperlink ref="B264:B264" r:id="Rb42375a696524e13" display="https://etf.dws.com//en-gb/LU0411075020-shortdax-x2-daily-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B265:B265" r:id="Rc08227772a4344fd" display="https://etf.dws.com//en-gb/LU0411075376-levdax-daily-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B266:B266" r:id="R8b281c1b307a48d7" display="https://etf.dws.com//en-gb/LU0411078552-s-p-500-2x-leveraged-daily-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B267:B267" r:id="R7baaf94f2f8a4817" display="https://etf.dws.com//en-gb/LU0411078636-s-p-500-2x-inverse-daily-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B268:B268" r:id="R9cc5e77527f84598" display="https://etf.dws.com//en-gb/LU0429458895-us-treasuries-1-3-ucits-etf-1d/"/>
-    <x:hyperlink ref="B269:B269" r:id="R11d3714047f54318" display="https://etf.dws.com//en-gb/LU0429459356-us-treasuries-ucits-etf-1d/"/>
-    <x:hyperlink ref="B270:B270" r:id="R9f5006d84e2049b2" display="https://etf.dws.com//en-gb/LU0429790743-bloomberg-commodity-swap-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B271:B271" r:id="R736c9599ce394d96" display="https://etf.dws.com//en-gb/LU0460391732-bloomberg-commodity-ex-agriculture-livestock-swap-ucits-etf-2c/"/>
-    <x:hyperlink ref="B272:B272" r:id="R9b231519c4bd45f2" display="https://etf.dws.com//en-gb/LU0460391906-bloomberg-commodity-ex-agriculture-livestock-swap-ucits-etf-3c-gbp-hedged/"/>
-    <x:hyperlink ref="B273:B273" r:id="R7d4e12d116a1407e" display="https://etf.dws.com//en-gb/LU0468896575-germany-government-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B274:B274" r:id="Rec48cc4b7bd54ecd" display="https://etf.dws.com//en-gb/LU0468897110-germany-government-bond-1-3-ucits-etf-1d/"/>
-    <x:hyperlink ref="B275:B275" r:id="Rf91a003ac1bf49b7" display="https://etf.dws.com//en-gb/LU0476289466-msci-mexico-ucits-etf-1c/"/>
-    <x:hyperlink ref="B276:B276" r:id="R52aea54b23674819" display="https://etf.dws.com//en-gb/LU0476289540-msci-canada-screened-ucits-etf-1c/"/>
-    <x:hyperlink ref="B277:B277" r:id="R73587414c03e442d" display="https://etf.dws.com//en-gb/LU0476289623-msci-indonesia-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B278:B278" r:id="R81d9cd4112fb479f" display="https://etf.dws.com//en-gb/LU0478205379-eur-corporate-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B279:B279" r:id="Rc64ec7a59f9a473d" display="https://etf.dws.com//en-gb/LU0478205965-eur-corporate-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B280:B280" r:id="R1b40bce8ad8246aa" display="https://etf.dws.com//en-gb/LU0484968812-eur-corporate-bond-sri-pab-ucits-etf-1d/"/>
-    <x:hyperlink ref="B281:B281" r:id="R35206aab174e40c8" display="https://etf.dws.com//en-gb/LU0484968903-eur-corporate-bond-sri-pab-ucits-etf-1c/"/>
-    <x:hyperlink ref="B282:B282" r:id="R858c2ed9cb2d4816" display="https://etf.dws.com//en-gb/LU0484969463-target-maturity-sept-2029-italy-and-spain-government-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B283:B283" r:id="Rd448073285414d47" display="https://etf.dws.com//en-gb/LU0486851024-msci-europe-value-ucits-etf-1c/"/>
-    <x:hyperlink ref="B284:B284" r:id="R1233112f364c42a1" display="https://etf.dws.com//en-gb/LU0489337690-ftse-developed-europe-real-estate-ucits-etf-1c/"/>
-    <x:hyperlink ref="B285:B285" r:id="R05ceb189b9e84c3f" display="https://etf.dws.com//en-gb/LU0490618542-s-p-500-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B286:B286" r:id="R0aea0e7b768446d8" display="https://etf.dws.com//en-gb/LU0494592974-australia-government-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B287:B287" r:id="R3bb680bc89b8416c" display="https://etf.dws.com//en-gb/LU0514694370-msci-malaysia-ucits-etf-1c/"/>
-    <x:hyperlink ref="B288:B288" r:id="R20e6fd8643e84c3e" display="https://etf.dws.com//en-gb/LU0514694701-msci-thailand-ucits-etf-1c/"/>
-    <x:hyperlink ref="B289:B289" r:id="R2e0516ecd4da441a" display="https://etf.dws.com//en-gb/LU0514695187-msci-india-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B290:B290" r:id="R8e4af0694ffd4a27" display="https://etf.dws.com//en-gb/LU0514695690-msci-china-ucits-etf-1c/"/>
-    <x:hyperlink ref="B291:B291" r:id="Rc5aaada953164663" display="https://etf.dws.com//en-gb/LU0524480265-iboxx-eurozone-government-bond-yield-plus-ucits-etf-1c/"/>
-    <x:hyperlink ref="B292:B292" r:id="Ra2cd04cd2d69463e" display="https://etf.dws.com//en-gb/LU0592215403-msci-philippines-ucits-etf-1c/"/>
-    <x:hyperlink ref="B293:B293" r:id="R53f620c726534c81" display="https://etf.dws.com//en-gb/LU0592216393-spain-ucits-etf-1c/"/>
-    <x:hyperlink ref="B294:B294" r:id="R91ffa5b38bbc4913" display="https://etf.dws.com//en-gb/LU0592217524-msci-africa-top-50-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B295:B295" r:id="R59386023f96b4a7b" display="https://etf.dws.com//en-gb/LU0613540268-italy-government-bond-0-1-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B296:B296" r:id="Rd5a2650b090e4187" display="https://etf.dws.com//en-gb/LU0614173549-eurozone-government-bond-1-3-ucits-etf-1d/"/>
-    <x:hyperlink ref="B297:B297" r:id="R16a1131b15db4a37" display="https://etf.dws.com//en-gb/LU0614173895-eurozone-government-bond-3-5-ucits-etf-1d/"/>
-    <x:hyperlink ref="B298:B298" r:id="R24734b824a844882" display="https://etf.dws.com//en-gb/LU0641006290-global-government-bond-ucits-etf-2d-gbp-hedged/"/>
-    <x:hyperlink ref="B299:B299" r:id="R3184d31948ff4286" display="https://etf.dws.com//en-gb/LU0641006456-global-government-bond-ucits-etf-3c-usd-hedged/"/>
-    <x:hyperlink ref="B300:B300" r:id="Rde4ecc4a19124436" display="https://etf.dws.com//en-gb/LU0641006613-global-government-bond-ucits-etf-4c-chf-hedged/"/>
-    <x:hyperlink ref="B301:B301" r:id="Rf0a742ba436d4995" display="https://etf.dws.com//en-gb/LU0641007009-global-inflation-linked-bond-ucits-etf-2c-usd-hedged/"/>
-    <x:hyperlink ref="B302:B302" r:id="Rea5f1bb574f54053" display="https://etf.dws.com//en-gb/LU0641007264-global-inflation-linked-bond-ucits-etf-3d-gbp-hedged/"/>
-    <x:hyperlink ref="B303:B303" r:id="R261a87f79c2f4779" display="https://etf.dws.com//en-gb/LU0641007421-global-inflation-linked-bond-ucits-etf-4d-chf-hedged/"/>
-    <x:hyperlink ref="B304:B304" r:id="R710956b0b75c4163" display="https://etf.dws.com//en-gb/LU0643975161-germany-government-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B305:B305" r:id="R4e581a2272cf458a" display="https://etf.dws.com//en-gb/LU0643975591-eurozone-government-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B306:B306" r:id="R07094ffba57048e4" display="https://etf.dws.com//en-gb/LU0659578842-msci-singapore-ucits-etf-1c/"/>
-    <x:hyperlink ref="B307:B307" r:id="R98626ca993b1460c" display="https://etf.dws.com//en-gb/LU0659579063-atx-ucits-etf-1c/"/>
-    <x:hyperlink ref="B308:B308" r:id="R600d9675cce34a2a" display="https://etf.dws.com//en-gb/LU0659579147-msci-pakistan-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B309:B309" r:id="Rfa0ea11aecdb4c2d" display="https://etf.dws.com//en-gb/LU0659579733-msci-world-swap-ucits-etf-4c-eur-hedged/"/>
-    <x:hyperlink ref="B310:B310" r:id="R07c3673932374a64" display="https://etf.dws.com//en-gb/LU0659580079-msci-japan-ucits-etf-4c-eur-hedged/"/>
-    <x:hyperlink ref="B311:B311" r:id="R7338d8af83c04d22" display="https://etf.dws.com//en-gb/LU0677077884-j-p-morgan-usd-emerging-markets-bond-ucits-etf-2d/"/>
-    <x:hyperlink ref="B312:B312" r:id="R474bbf23684442b9" display="https://etf.dws.com//en-gb/LU0690964092-global-government-bond-ucits-etf-1d-eur-hedged/"/>
-    <x:hyperlink ref="B313:B313" r:id="R2509fbc145f048ff" display="https://etf.dws.com//en-gb/LU0779800910-csi300-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B314:B314" r:id="Rb8d5908649a745fb" display="https://etf.dws.com//en-gb/LU0838780707-ftse-100-ucits-etf-1c/"/>
-    <x:hyperlink ref="B315:B315" r:id="Rf86ecbffcf4745e4" display="https://etf.dws.com//en-gb/LU0838782315-dax-esg-screened-ucits-etf-1d/"/>
-    <x:hyperlink ref="B316:B316" r:id="R623e07bba15f4fe0" display="https://etf.dws.com//en-gb/LU0839027447-nikkei-225-ucits-etf-1d/"/>
-    <x:hyperlink ref="B317:B317" r:id="R281cd84b12c54b32" display="https://etf.dws.com//en-gb/LU0846194776-msci-emu-ucits-etf-1d/"/>
-    <x:hyperlink ref="B318:B318" r:id="R51423d2a9d6f452b" display="https://etf.dws.com//en-gb/LU0875160326-harvest-csi300-ucits-etf-1d/"/>
-    <x:hyperlink ref="B319:B319" r:id="R692cf5fc8033424e" display="https://etf.dws.com//en-gb/LU0908508731-global-government-bond-ucits-etf-5c/"/>
-    <x:hyperlink ref="B320:B320" r:id="R8365ef61cf4c4c54" display="https://etf.dws.com//en-gb/LU0908508814-global-inflation-linked-bond-ucits-etf-5c/"/>
-    <x:hyperlink ref="B321:B321" r:id="Ra93b3699187041be" display="https://etf.dws.com//en-gb/LU0925589839-iboxx-eurozone-government-bond-yield-plus-1-3-ucits-etf-1c/"/>
-    <x:hyperlink ref="B322:B322" r:id="Rf36b0f18e5454c67" display="https://etf.dws.com//en-gb/LU0927735406-msci-japan-ucits-etf-2d-usd-hedged/"/>
-    <x:hyperlink ref="B323:B323" r:id="R048114ef8de147a6" display="https://etf.dws.com//en-gb/LU0942970103-esg-global-aggregate-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B324:B324" r:id="Rda002071d746432a" display="https://etf.dws.com//en-gb/LU0942970285-esg-global-aggregate-bond-ucits-etf-2c-usd-hedged/"/>
-    <x:hyperlink ref="B325:B325" r:id="Rbdfb7db7f6e64061" display="https://etf.dws.com//en-gb/LU0942970368-esg-global-aggregate-bond-ucits-etf-3d-gbp-hedged/"/>
-    <x:hyperlink ref="B326:B326" r:id="R02795e576b304eeb" display="https://etf.dws.com//en-gb/LU0942970442-esg-global-aggregate-bond-ucits-etf-4c-chf-hedged/"/>
-    <x:hyperlink ref="B327:B327" r:id="Rc7f8d64c104a42c4" display="https://etf.dws.com//en-gb/LU0942970798-esg-global-aggregate-bond-ucits-etf-5c-eur-hedged/"/>
-    <x:hyperlink ref="B328:B328" r:id="R1ce71a883944415a" display="https://etf.dws.com//en-gb/LU0943504760-switzerland-ucits-etf-1c/"/>
-    <x:hyperlink ref="B329:B329" r:id="R54585639ebff480e" display="https://etf.dws.com//en-gb/LU0952581584-japan-government-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B330:B330" r:id="R676399e4c93f4387" display="https://etf.dws.com//en-gb/LU0962071741-iboxx-eurozone-government-bond-yield-plus-ucits-etf-1d/"/>
-    <x:hyperlink ref="B331:B331" r:id="R0d3a60ff449f48cd" display="https://etf.dws.com//en-gb/LU0962078753-global-inflation-linked-bond-ucits-etf-1d-eur-hedged/"/>
-    <x:hyperlink ref="B332:B332" r:id="R86d851325197469f" display="https://etf.dws.com//en-gb/LU0994505336-spain-ucits-etf-1d/"/>
-    <x:hyperlink ref="B333:B333" r:id="Rb8dd8922761f4942" display="https://etf.dws.com//en-gb/LU1094612022-harvest-china-government-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B334:B334" r:id="Rf316f4505928479a" display="https://etf.dws.com//en-gb/LU1109939865-rolling-target-maturity-sept-2027-eur-high-yield-ucits-etf-1d/"/>
-    <x:hyperlink ref="B335:B335" r:id="R998310a849814175" display="https://etf.dws.com//en-gb/LU1109941689-rolling-target-maturity-sept-2027-eur-high-yield-ucits-etf-1c/"/>
-    <x:hyperlink ref="B336:B336" r:id="R9bcf35cbb674458c" display="https://etf.dws.com//en-gb/LU1109942653-eur-high-yield-corporate-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B337:B337" r:id="Rdbcf3a7a9ee141f8" display="https://etf.dws.com//en-gb/LU1109943388-eur-high-yield-corporate-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B338:B338" r:id="R9bf9559accb64c77" display="https://etf.dws.com//en-gb/LU1127514245-msci-emu-ucits-etf-1c-usd-hedged/"/>
-    <x:hyperlink ref="B339:B339" r:id="R6a222a7f19024a31" display="https://etf.dws.com//en-gb/LU1127516455-msci-emu-ucits-etf-2c-gbp-hedged/"/>
-    <x:hyperlink ref="B340:B340" r:id="Rbe510119c7af48b0" display="https://etf.dws.com//en-gb/LU1184092051-msci-europe-ucits-etf-2c-usd-hedged/"/>
-    <x:hyperlink ref="B341:B341" r:id="R44e01935e1484c38" display="https://etf.dws.com//en-gb/LU1215827756-msci-japan-ucits-etf-7c-chf-hedged/"/>
-    <x:hyperlink ref="B342:B342" r:id="R1ead12fb11424cbb" display="https://etf.dws.com//en-gb/LU1215828218-msci-emu-ucits-etf-3c-chf-hedged/"/>
-    <x:hyperlink ref="B343:B343" r:id="R0ef9cd3c34d04cb0" display="https://etf.dws.com//en-gb/LU1221100792-dax-esg-screened-ucits-etf-2c-usd-hedged/"/>
-    <x:hyperlink ref="B344:B344" r:id="R9748a96942994acb" display="https://etf.dws.com//en-gb/LU1221102491-dax-esg-screened-ucits-etf-4c-chf-hedged/"/>
-    <x:hyperlink ref="B345:B345" r:id="R17f491ef056d49cd" display="https://etf.dws.com//en-gb/LU1242369327-msci-europe-ucits-etf-1d/"/>
-    <x:hyperlink ref="B346:B346" r:id="Re6a4430a0a744e62" display="https://etf.dws.com//en-gb/LU1310477036-harvest-csi-a500-ucits-etf-1d/"/>
-    <x:hyperlink ref="B347:B347" r:id="Rfa06a011c9414054" display="https://etf.dws.com//en-gb/LU1349386927-dax-ucits-etf-1d/"/>
-    <x:hyperlink ref="B348:B348" r:id="Rba3cbb9969e3445b" display="https://etf.dws.com//en-gb/LU1399300455-us-treasuries-ucits-etf-2d-eur-hedged/"/>
-    <x:hyperlink ref="B349:B349" r:id="R018750b3f8024bf4" display="https://etf.dws.com//en-gb/LU1772333404-stoxx-europe-600-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B350:B350" r:id="R06ccc37ba7594c03" display="https://etf.dws.com//en-gb/LU1875395870-nikkei-225-ucits-etf-2d-eur-hedged/"/>
-    <x:hyperlink ref="B351:B351" r:id="Rc5461ce497524ed7" display="https://etf.dws.com//en-gb/LU1920015440-j-p-morgan-usd-emerging-markets-bond-ucits-etf-2c/"/>
-    <x:hyperlink ref="B352:B352" r:id="R754022b0dcdb483e" display="https://etf.dws.com//en-gb/LU1920015523-us-treasuries-1-3-ucits-etf-1c/"/>
-    <x:hyperlink ref="B353:B353" r:id="Rec26d4b456c341c4" display="https://etf.dws.com//en-gb/LU1920015796-us-treasuries-ucits-etf-1c/"/>
-    <x:hyperlink ref="B354:B354" r:id="R116a658245844b77" display="https://etf.dws.com//en-gb/LU2009147591-eurozone-government-bond-ucits-etf-2c-usd-hedged/"/>
-    <x:hyperlink ref="B355:B355" r:id="Rf46964348307450d" display="https://etf.dws.com//en-gb/LU2009147757-s-p-500-swap-ucits-etf-1d/"/>
-    <x:hyperlink ref="B356:B356" r:id="R6df25c2fedf04126" display="https://etf.dws.com//en-gb/LU2158769930-j-p-morgan-em-local-government-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B357:B357" r:id="R8895f94adffe420a" display="https://etf.dws.com//en-gb/LU2178481649-eur-corporate-bond-short-duration-sri-pab-ucits-etf-1c/"/>
-    <x:hyperlink ref="B358:B358" r:id="Rbf46b215e9524d64" display="https://etf.dws.com//en-gb/LU2196470426-nikkei-225-ucits-etf-1c/"/>
-    <x:hyperlink ref="B359:B359" r:id="R2164c4623f3b41ca" display="https://etf.dws.com//en-gb/LU2196472984-s-p-500-swap-ucits-etf-5c-eur-hedged/"/>
-    <x:hyperlink ref="B360:B360" r:id="R1ecc5e3bdc0d44c6" display="https://etf.dws.com//en-gb/LU2196473016-s-p-500-swap-ucits-etf-7c-gbp-hedged/"/>
-    <x:hyperlink ref="B361:B361" r:id="R88405c21a28c47da" display="https://etf.dws.com//en-gb/LU2263803533-msci-world-swap-ucits-etf-1d/"/>
-    <x:hyperlink ref="B362:B362" r:id="Ra9ccfaf8f5394dbe" display="https://etf.dws.com//en-gb/LU2278080713-bloomberg-commodity-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B363:B363" r:id="R62bd93b36fc24669" display="https://etf.dws.com//en-gb/LU2296661775-msci-em-asia-screened-swap-ucits-etf-1d/"/>
-    <x:hyperlink ref="B364:B364" r:id="R94c3e868c64e4e22" display="https://etf.dws.com//en-gb/LU2361257269-j-p-morgan-usd-emerging-markets-bond-ucits-etf-1d-eur-hedged/"/>
-    <x:hyperlink ref="B365:B365" r:id="Rc56b6078f4f54300" display="https://etf.dws.com//en-gb/LU2376679564-harvest-msci-china-tech-100-ucits-etf-1c/"/>
-    <x:hyperlink ref="B366:B366" r:id="Rf5d8fb71f3e842c3" display="https://etf.dws.com//en-gb/LU2385068163-esg-global-government-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B367:B367" r:id="R5b7f328435fc43ac" display="https://etf.dws.com//en-gb/LU2385068247-esg-global-government-bond-ucits-etf-2d-gbp-hedged/"/>
-    <x:hyperlink ref="B368:B368" r:id="R3cf893d777924221" display="https://etf.dws.com//en-gb/LU2385068320-esg-global-government-bond-ucits-etf-3d-usd-hedged/"/>
-    <x:hyperlink ref="B369:B369" r:id="R3855d6a916414c91" display="https://etf.dws.com//en-gb/LU2385068593-esg-global-government-bond-ucits-etf-4d-eur-hedged/"/>
-    <x:hyperlink ref="B370:B370" r:id="R9f4e8c372d3e4e25" display="https://etf.dws.com//en-gb/LU2456436083-msci-china-ucits-etf-1d/"/>
-    <x:hyperlink ref="B371:B371" r:id="Rf5311309406b45dc" display="https://etf.dws.com//en-gb/LU2462217071-esg-global-government-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B372:B372" r:id="Rae02b4934492478f" display="https://etf.dws.com//en-gb/LU2468423459-esg-eurozone-government-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B373:B373" r:id="R384274723c2d4ed4" display="https://etf.dws.com//en-gb/LU2469465822-msci-china-a-screened-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B374:B374" r:id="Rcddeeed524aa40b8" display="https://etf.dws.com//en-gb/LU2504532131-tips-us-inflation-linked-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B375:B375" r:id="R44b592872cc44197" display="https://etf.dws.com//en-gb/LU2504532487-eurozone-government-green-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B376:B376" r:id="R5300cb733dd44694" display="https://etf.dws.com//en-gb/LU2504537445-eurozone-government-bond-esg-tilted-ucits-etf-1d/"/>
-    <x:hyperlink ref="B377:B377" r:id="Re2db4e29bf274a51" display="https://etf.dws.com//en-gb/LU2523865728-eurozone-government-bond-7-10-ucits-etf-1d-gbp-hedged/"/>
-    <x:hyperlink ref="B378:B378" r:id="R65b8949919f14bc8" display="https://etf.dws.com//en-gb/LU2523865991-eurozone-government-bond-7-10-ucits-etf-2c-usd-hedged/"/>
-    <x:hyperlink ref="B379:B379" r:id="R39ed96ad84fc4b95" display="https://etf.dws.com//en-gb/LU2523866023-eurozone-government-bond-ucits-etf-2d-gbp-hedged/"/>
-    <x:hyperlink ref="B380:B380" r:id="R7c6eaa70c37a4590" display="https://etf.dws.com//en-gb/LU2523866296-germany-government-bond-ucits-etf-2d-gbp-hedged/"/>
-    <x:hyperlink ref="B381:B381" r:id="R8c3be1a631a4478f" display="https://etf.dws.com//en-gb/LU2523866379-germany-government-bond-ucits-etf-2c-usd-hedged/"/>
-    <x:hyperlink ref="B382:B382" r:id="Rf7a698d187ea4a03" display="https://etf.dws.com//en-gb/LU2552296563-iboxx-eurozone-government-bond-yield-plus-1-3-ucits-etf-2d/"/>
-    <x:hyperlink ref="B383:B383" r:id="R6922adfb2ca946be" display="https://etf.dws.com//en-gb/LU2581375073-msci-usa-swap-ucits-etf-1d/"/>
-    <x:hyperlink ref="B384:B384" r:id="R2979a8cc81864db2" display="https://etf.dws.com//en-gb/LU2581375156-stoxx-europe-600-ucits-etf-1d/"/>
-    <x:hyperlink ref="B385:B385" r:id="R5a728bc3a5a64ba0" display="https://etf.dws.com//en-gb/LU2581375230-msci-japan-ucits-etf-1d/"/>
-    <x:hyperlink ref="B386:B386" r:id="Rfc96b8e3a5b64dbd" display="https://etf.dws.com//en-gb/LU2606231335-eurozone-government-bond-3-5-ucits-etf-2c-usd-hedged/"/>
-    <x:hyperlink ref="B387:B387" r:id="Reb15512f135b48df" display="https://etf.dws.com//en-gb/LU2606231418-eurozone-government-bond-3-5-ucits-etf-2d-gbp-hedged/"/>
-    <x:hyperlink ref="B388:B388" r:id="Ra83ba568f34e495b" display="https://etf.dws.com//en-gb/LU2610432036-us-treasuries-ucits-etf-2c-gbp-hedged/"/>
-    <x:hyperlink ref="B389:B389" r:id="R4dce939db5d74049" display="https://etf.dws.com//en-gb/LU2641054122-eurozone-government-bond-0-1-ucits-etf-1c/"/>
-    <x:hyperlink ref="B390:B390" r:id="R415a0d7f0d384f4f" display="https://etf.dws.com//en-gb/LU2641054551-germany-government-bond-0-1-ucits-etf-1c/"/>
-    <x:hyperlink ref="B391:B391" r:id="R9bb214a013f942ac" display="https://etf.dws.com//en-gb/LU2662649412-us-treasuries-10-ucits-etf-1d/"/>
-    <x:hyperlink ref="B392:B392" r:id="R8830d7e3e02e48bf" display="https://etf.dws.com//en-gb/LU2662649503-us-treasuries-3-7-ucits-etf-1d/"/>
-    <x:hyperlink ref="B393:B393" r:id="R3ae4d1cf16044c97" display="https://etf.dws.com//en-gb/LU2662649685-us-treasuries-7-10-ucits-etf-1d/"/>
-    <x:hyperlink ref="B394:B394" r:id="R478576b142d64c84" display="https://etf.dws.com//en-gb/LU2673522830-target-maturity-sept-2027-eur-corporate-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B395:B395" r:id="R3bb8a8fa60244e16" display="https://etf.dws.com//en-gb/LU2673522913-target-maturity-sept-2029-eur-corporate-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B396:B396" r:id="R1a8b1dd14b084de6" display="https://etf.dws.com//en-gb/LU2673523051-target-maturity-sept-2033-eur-corporate-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B397:B397" r:id="Ref67b69e2dc143bd" display="https://etf.dws.com//en-gb/LU2673523135-target-maturity-sept-2031-eur-corporate-bond-ucits-etf-1c/"/>
-    <x:hyperlink ref="B398:B398" r:id="R7bd81a20ff044e1f" display="https://etf.dws.com//en-gb/LU2673523218-target-maturity-sept-2027-eur-corporate-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B399:B399" r:id="R8023874ea1fc48d6" display="https://etf.dws.com//en-gb/LU2673523309-target-maturity-sept-2029-eur-corporate-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B400:B400" r:id="R59589b56ff104835" display="https://etf.dws.com//en-gb/LU2673523481-target-maturity-sept-2031-eur-corporate-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B401:B401" r:id="R0a744cb539c34a05" display="https://etf.dws.com//en-gb/LU2673523564-target-maturity-sept-2033-eur-corporate-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B402:B402" r:id="Ree654cfc02a34325" display="https://etf.dws.com//en-gb/LU2675291913-msci-emerging-markets-swap-ucits-etf-1d/"/>
-    <x:hyperlink ref="B403:B403" r:id="Rb596717d134c4be4" display="https://etf.dws.com//en-gb/LU2755521270-msci-pacific-ex-japan-ucits-etf-1d/"/>
-    <x:hyperlink ref="B404:B404" r:id="R9b842ce24d7d45a8" display="https://etf.dws.com//en-gb/LU2788421340-csi500-swap-ucits-etf-1c/"/>
-    <x:hyperlink ref="B405:B405" r:id="R6c3d7bedb2b24930" display="https://etf.dws.com//en-gb/LU2809864296-target-maturity-sept-2030-eur-corporate-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B406:B406" r:id="Ra036ad87dda842d0" display="https://etf.dws.com//en-gb/LU2809864452-target-maturity-sept-2032-eur-corporate-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B407:B407" r:id="Rd828b0a300474918" display="https://etf.dws.com//en-gb/LU2809864619-target-maturity-sept-2034-eur-corporate-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B408:B408" r:id="R939095211f3b4a6f" display="https://etf.dws.com//en-gb/LU2810185665-target-maturity-sept-2028-eur-corporate-bond-ucits-etf-1d/"/>
-    <x:hyperlink ref="B409:B409" r:id="Refbf84f491724249" display="https://etf.dws.com//en-gb/LU2859297330-world-small-cap-green-tech-innovators-ucits-etf-1c/"/>
-    <x:hyperlink ref="B410:B410" r:id="R36c5d346994d4d6a" display="https://etf.dws.com//en-gb/LU2859392081-world-green-tech-innovators-ucits-etf-1c/"/>
-    <x:hyperlink ref="B411:B411" r:id="Ree2059485abc4233" display="https://etf.dws.com//en-gb/LU2903252349-scalable-msci-ac-world-xtrackers-ucits-etf-1c/"/>
-    <x:hyperlink ref="B412:B412" r:id="Rb9e7c11af8b64ab6" display="https://etf.dws.com//en-gb/LU2928641757-msci-taiwan-ucits-etf-1d/"/>
-    <x:hyperlink ref="B413:B413" r:id="R84bb71dc7b8048e5" display="https://etf.dws.com//en-gb/LU3003217554-eurozone-government-bond-1-3-ucits-etf-2c-usd-hedged/"/>
-    <x:hyperlink ref="B414:B414" r:id="Rdab3e86b88c24617" display="https://etf.dws.com//en-gb/LU3003217638-eurozone-government-bond-1-3-ucits-etf-2d-gbp-hedged/"/>
-    <x:hyperlink ref="B415:B415" r:id="R1311b255e45949de" display="https://etf.dws.com//en-gb/LU3003217711-eurozone-government-bond-5-7-ucits-etf-2c-usd-hedged/"/>
-    <x:hyperlink ref="B416:B416" r:id="Rf651b8c68d87464c" display="https://etf.dws.com//en-gb/LU3003217984-eurozone-government-bond-5-7-ucits-etf-1d-gbp-hedged/"/>
-    <x:hyperlink ref="B417:B417" r:id="Reeb9e1963e8b4462" display="https://etf.dws.com//en-gb/LU3003218016-australia-government-bond-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B418:B418" r:id="R5e001191b1e94867" display="https://etf.dws.com//en-gb/LU3003218107-australia-government-bond-ucits-etf-3c-usd-hedged/"/>
-    <x:hyperlink ref="B419:B419" r:id="R83a167600adf46db" display="https://etf.dws.com//en-gb/LU3003218362-australia-government-bond-ucits-etf-1d-gbp-hedged/"/>
-    <x:hyperlink ref="B420:B420" r:id="Rbaba7842653142d9" display="https://etf.dws.com//en-gb/LU3003218446-japan-government-bond-ucits-etf-2c-eur-hedged/"/>
-    <x:hyperlink ref="B421:B421" r:id="Rfc27b250f1474ba4" display="https://etf.dws.com//en-gb/LU3003218792-japan-government-bond-ucits-etf-3c-usd-hedged/"/>
-    <x:hyperlink ref="B422:B422" r:id="R407ad69abd1b47e8" display="https://etf.dws.com//en-gb/LU3003218958-japan-government-bond-ucits-etf-2d-gbp-hedged/"/>
-    <x:hyperlink ref="B423:B423" r:id="Rd9272f91d1ec4ffb" display="https://etf.dws.com//en-gb/LU3061478973-europe-defence-technologies-ucits-etf-1c/"/>
-    <x:hyperlink ref="B424:B424" r:id="Ra5383e7b58434d44" display="https://etf.dws.com//en-gb/LU3116008346-diversified-portfolio-20-equity-ucits-etf-1c/"/>
-    <x:hyperlink ref="B425:B425" r:id="R05255a9980f64ca9" display="https://etf.dws.com//en-gb/LU3116008429-diversified-portfolio-40-equity-ucits-etf-1c/"/>
-    <x:hyperlink ref="B426:B426" r:id="R5bc88106dc6d4b0c" display="https://etf.dws.com//en-gb/LU3116008692-diversified-portfolio-60-equity-ucits-etf-1c/"/>
-    <x:hyperlink ref="B427:B427" r:id="Ra4428e62adad4cc2" display="https://etf.dws.com//en-gb/LU3116008775-diversified-portfolio-80-equity-ucits-etf-1c/"/>
-    <x:hyperlink ref="B428:B428" r:id="R229f886f300e4d49" display="https://etf.dws.com//en-gb/LU3121019551-global-government-bond-ucits-etf-3d-chf-hedged/"/>
-    <x:hyperlink ref="B429:B429" r:id="R7ade6a1f0c9a44cd" display="https://etf.dws.com//en-gb/LU3123443510-salam-usd-global-aggregate-sukuk-ucits-etf-1d/"/>
-    <x:hyperlink ref="B430:B430" r:id="Rd21066365a9447d1" display="https://etf.dws.com//en-gb/LU3184977026-msci-world-swap-ucits-etf-ic-gbp-unlisted/"/>
-    <x:hyperlink ref="B431:B431" r:id="R2785de30262449a5" display="https://etf.dws.com//en-gb/LU3184977299-msci-europe-ucits-etf-ic-eur-unlisted/"/>
-    <x:hyperlink ref="B432:B432" r:id="Rcf76fe2d923d46bd" display="https://etf.dws.com//en-gb/LU3184977372-msci-usa-swap-ucits-etf-ic-gbp-unlisted/"/>
-    <x:hyperlink ref="B433:B433" r:id="R7b679b6ef084400b" display="https://etf.dws.com//en-gb/LU3184977455-msci-emerging-markets-swap-ucits-etf-ic-gbp-unlisted/"/>
-    <x:hyperlink ref="B434:B434" r:id="Raef3f3d7659742b1" display="https://etf.dws.com//en-gb/LU3184977612-s-p-500-swap-ucits-etf-ic-gbp-unlisted/"/>
-    <x:hyperlink ref="B435:B435" r:id="Rf8512baaaff343d1" display="https://etf.dws.com//en-gb/LU3184977703-ftse-100-ucits-etf-ic-gbp-unlisted/"/>
-    <x:hyperlink ref="B436:B436" r:id="Rc1aca96dd6d64432" display="https://etf.dws.com//en-gb/LU3198621024-s-p-500-swap-ucits-etf-ic-usd-unlisted/"/>
-    <x:hyperlink ref="B437:B437" r:id="Ree9bed38992c465c" display="https://etf.dws.com//en-gb/LU3284391318-global-government-bond-ucits-etf-4d/"/>
-    <x:hyperlink ref="B438:B438" r:id="Rbcd544d50f53405a" display="https://etf.dws.com//en-gb/LU3313127113-eurozone-government-bond-ucits-etf-ic-eur-unlisted/"/>
-    <x:hyperlink ref="B439:B439" r:id="Ra273d3c3a2e340de" display="https://etf.dws.com//en-gb/LU3353962601-msci-world-swap-ucits-etf-ic-eur-unlisted/"/>
-    <x:hyperlink ref="B440:B440" r:id="Rdb099094bc534493" display="https://etf.dws.com//en-gb/LU3353962783-s-p-500-swap-ucits-etf-ic-eur-unlisted/"/>
-    <x:hyperlink ref="B441:B441" r:id="R32479cc46663404e" display="https://etf.dws.com//en-gb/LU3353962866-stoxx-global-select-dividend-100-swap-ucits-etf-ic-usd-unlisted/"/>
-    <x:hyperlink ref="B442:B442" r:id="R149b0fae323546e8" display="https://etf.dws.com//en-gb/LU3353962940-stoxx-europe-600-ucits-etf-ic-eur-unlisted/"/>
-    <x:hyperlink ref="B443:B443" r:id="Rd41689bef02147a0" display="https://etf.dws.com//en-gb/LU3370249040-bloomberg-commodity-swap-ucits-etf-3c-gbp-hedged/"/>
-    <x:hyperlink ref="B444:B444" r:id="R31a3ee0e76064b3d" display="https://etf.dws.com//en-gb/LU3375213041-msci-world-swap-ucits-etf-ic-usd-unlisted/"/>
+    <x:hyperlink ref="B8:B8" r:id="R6e7807c7f60e4fe8" display="https://etf.dws.com//en-gb/IE00002ZKAP0-europe-equity-enhanced-active-ucits-etf-1c/"/>
+    <x:hyperlink ref="B9:B9" r:id="R7be2330456f1433b" display="https://etf.dws.com//en-gb/IE00004DJ199-msci-world-swap-ii-ucits-etf-1d/"/>
+    <x:hyperlink ref="B10:B10" r:id="R5d6ad2338e24461e" display="https://etf.dws.com//en-gb/IE0000K7HU41-msci-usa-information-technology-ucits-etf-1c/"/>
+    <x:hyperlink ref="B11:B11" r:id="R10beec56848c4fc7" display="https://etf.dws.com//en-gb/IE0000MMQ5M5-msci-usa-esg-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B12:B12" r:id="Refe3a16194664aa1" display="https://etf.dws.com//en-gb/IE0001JH5CB4-europe-net-zero-pathway-paris-aligned-ucits-etf-1c/"/>
+    <x:hyperlink ref="B13:B13" r:id="R7bfbb66bf39a4afa" display="https://etf.dws.com//en-gb/IE0001TLQX55-s-p-500-garp-ucits-etf-1c/"/>
+    <x:hyperlink ref="B14:B14" r:id="Rddf690b04fc64af5" display="https://etf.dws.com//en-gb/IE00028H9QJ8-usd-corporate-green-bond-ucits-etf-1c-eur-hedged/"/>
+    <x:hyperlink ref="B15:B15" r:id="R518057d3c5944136" display="https://etf.dws.com//en-gb/IE0002EI5AG0-s-p-500-equal-weight-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B16:B16" r:id="R666a193c35a94e15" display="https://etf.dws.com//en-gb/IE0002GFATQ6-s-p-500-equal-weight-ucits-etf-3c-chf-hedged/"/>
+    <x:hyperlink ref="B17:B17" r:id="Rd4a4f28b3d4746bc" display="https://etf.dws.com//en-gb/IE0002PGSLZ5-us-equity-enhanced-active-ucits-etf-1c/"/>
+    <x:hyperlink ref="B18:B18" r:id="Rf5729d18022447af" display="https://etf.dws.com//en-gb/IE0002ZM3JI1-usa-net-zero-pathway-paris-aligned-ucits-etf-1c/"/>
+    <x:hyperlink ref="B19:B19" r:id="Rc559fda7996e4c26" display="https://etf.dws.com//en-gb/IE00036F4K40-msci-global-sdg-3-good-health-ucits-etf-1c/"/>
+    <x:hyperlink ref="B20:B20" r:id="R615ab5551e4446f5" display="https://etf.dws.com//en-gb/IE0003NQ0IY5-msci-world-quality-esg-ucits-etf-1c/"/>
+    <x:hyperlink ref="B21:B21" r:id="Re3b1e03cf5dc47ac" display="https://etf.dws.com//en-gb/IE0003W9O921-usd-corporate-green-bond-ucits-etf-2c/"/>
+    <x:hyperlink ref="B22:B22" r:id="R5a1e67fddf8d4524" display="https://etf.dws.com//en-gb/IE000472H9T4-nasdaq-100-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B23:B23" r:id="R10c2f529c52a45fa" display="https://etf.dws.com//en-gb/IE0004KLW911-esg-usd-emerging-markets-bond-quality-weighted-ucits-etf-1c/"/>
+    <x:hyperlink ref="B24:B24" r:id="Rece2450e2c874e96" display="https://etf.dws.com//en-gb/IE0004MFRED4-s-p-500-equal-weight-scored-screened-ucits-etf-1c/"/>
+    <x:hyperlink ref="B25:B25" r:id="Rf227fc2ca3084164" display="https://etf.dws.com//en-gb/IE0004ZJGWT9-msci-europe-esg-ucits-etf-1d/"/>
+    <x:hyperlink ref="B26:B26" r:id="Rcaacc740bbc64cc0" display="https://etf.dws.com//en-gb/IE0005E47AH7-msci-global-sdg-9-industry-innovation-infrastructure-ucits-etf-1c/"/>
+    <x:hyperlink ref="B27:B27" r:id="Rd925b8d5a7a24112" display="https://etf.dws.com//en-gb/IE0006FDYJF8-msci-japan-climate-transition-ucits-etf-1d/"/>
+    <x:hyperlink ref="B28:B28" r:id="Rdd36ebdaeab943e2" display="https://etf.dws.com//en-gb/IE0006FFX5U1-msci-innovation-ucits-etf-1c/"/>
+    <x:hyperlink ref="B29:B29" r:id="R74d56f0aef5f44d5" display="https://etf.dws.com//en-gb/IE0006GNB732-eur-high-yield-corporate-bond-sri-pab-ucits-etf-1c/"/>
+    <x:hyperlink ref="B30:B30" r:id="R64b22b8662004985" display="https://etf.dws.com//en-gb/IE0006I3NZF8-msci-usa-consumer-discretionary-ucits-etf-1c/"/>
+    <x:hyperlink ref="B31:B31" r:id="Rb1897280453e4da6" display="https://etf.dws.com//en-gb/IE0006WW1TQ4-msci-world-ex-usa-ucits-etf-1c/"/>
+    <x:hyperlink ref="B32:B32" r:id="Rb3df7874d120457d" display="https://etf.dws.com//en-gb/IE0006YM7D84-usd-high-yield-corporate-bond-screened-ucits-etf-1c/"/>
+    <x:hyperlink ref="B33:B33" r:id="Rbe69a870b22b418d" display="https://etf.dws.com//en-gb/IE00074JLU02-japan-net-zero-pathway-paris-aligned-ucits-etf-1c/"/>
+    <x:hyperlink ref="B34:B34" r:id="Ra476cfd238ab4888" display="https://etf.dws.com//en-gb/IE0007ULOZS8-s-p-500-scored-screened-ucits-etf-1c/"/>
+    <x:hyperlink ref="B35:B35" r:id="R75a05c6ab4844497" display="https://etf.dws.com//en-gb/IE0007WJ6B10-msci-global-clean-water-sanitation-ucits-etf-1c/"/>
+    <x:hyperlink ref="B36:B36" r:id="R7ca1dfc7b80b45f7" display="https://etf.dws.com//en-gb/IE0008YN0OY8-msci-world-minimum-volatility-esg-ucits-etf-1c/"/>
+    <x:hyperlink ref="B37:B37" r:id="Rd24cc5d055814a37" display="https://etf.dws.com//en-gb/IE00094GSCQ4-world-equity-enhanced-active-ucits-etf-1c/"/>
+    <x:hyperlink ref="B38:B38" r:id="R07b15efd02b44afb" display="https://etf.dws.com//en-gb/IE0009KLWT21-msci-world-ucits-etf-3c-chf-hedged/"/>
+    <x:hyperlink ref="B39:B39" r:id="Rc1e097d5cf444ea1" display="https://etf.dws.com//en-gb/IE000BO2Y0T8-msci-nordic-ucits-etf-1c/"/>
+    <x:hyperlink ref="B40:B40" r:id="Rf9976babbe9c4255" display="https://etf.dws.com//en-gb/IE000CXLGK86-s-p-500-equal-weight-ucits-etf-2d/"/>
+    <x:hyperlink ref="B41:B41" r:id="Rc48604125989483a" display="https://etf.dws.com//en-gb/IE000DNSAS54-msci-emerging-markets-climate-transition-ucits-etf-1c/"/>
+    <x:hyperlink ref="B42:B42" r:id="R35a5790869004c1e" display="https://etf.dws.com//en-gb/IE000DVHJV46-s-p-500-market-leaders-ucits-etf-1c/"/>
+    <x:hyperlink ref="B43:B43" r:id="Rd81f824cf9d94645" display="https://etf.dws.com//en-gb/IE000E0V65D8-world-biodiversity-focus-sri-ucits-etf-1c/"/>
+    <x:hyperlink ref="B44:B44" r:id="R09f717176b9b4f98" display="https://etf.dws.com//en-gb/IE000E4BATC9-msci-world-esg-ucits-etf-1d/"/>
+    <x:hyperlink ref="B45:B45" r:id="R02cc5d90901a44d9" display="https://etf.dws.com//en-gb/IE000ER61U30-msci-europe-small-cap-esg-ucits-etf-1c/"/>
+    <x:hyperlink ref="B46:B46" r:id="R0e2e0053116043fa" display="https://etf.dws.com//en-gb/IE000EVOVOG1-msci-usa-positioning-screened-ucits-etf-1d/"/>
+    <x:hyperlink ref="B47:B47" r:id="Rb3c13f92cce644d3" display="https://etf.dws.com//en-gb/IE000EXUE0G2-nasdaq-100-swap-ucits-etf-1d/"/>
+    <x:hyperlink ref="B48:B48" r:id="Rbd19047117f447f4" display="https://etf.dws.com//en-gb/IE000F04HGE5-floating-rate-notes-active-ucits-etf-1c/"/>
+    <x:hyperlink ref="B49:B49" r:id="R4cc985bf26714736" display="https://etf.dws.com//en-gb/IE000F354Q61-msci-world-small-cap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B50:B50" r:id="R43fa23cdca874925" display="https://etf.dws.com//en-gb/IE000FL46JJ1-s-p-500-equal-weight-swap-ucits-etf-1d/"/>
+    <x:hyperlink ref="B51:B51" r:id="R012d0dd9d1da444a" display="https://etf.dws.com//en-gb/IE000FO05UG4-s-p-500-swap-ii-ucits-etf-1d/"/>
+    <x:hyperlink ref="B52:B52" r:id="R6664405fbbf14a7a" display="https://etf.dws.com//en-gb/IE000FO1A5D1-s-p-500-equal-weight-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B53:B53" r:id="Ra14fcb6337184554" display="https://etf.dws.com//en-gb/IE000FW16TX1-msci-usa-swap-ii-ucits-etf-1d/"/>
+    <x:hyperlink ref="B54:B54" r:id="Rfc41230744e649bb" display="https://etf.dws.com//en-gb/IE000GF6QTP6-s-p-500-equal-weight-scored-screened-ucits-etf-3c-chf-hedged/"/>
+    <x:hyperlink ref="B55:B55" r:id="R51a1e1209e514035" display="https://etf.dws.com//en-gb/IE000GWA2J58-msci-emerging-markets-ucits-etf-1d/"/>
+    <x:hyperlink ref="B56:B56" r:id="R71ac5805f8a445fb" display="https://etf.dws.com//en-gb/IE000GYDNJS5-msci-usa-climate-transition-ucits-etf-1d/"/>
+    <x:hyperlink ref="B57:B57" r:id="R84bb3ff2d8864fc1" display="https://etf.dws.com//en-gb/IE000HT7E0B1-nordic-net-zero-pathway-paris-aligned-ucits-etf-1c/"/>
+    <x:hyperlink ref="B58:B58" r:id="R336b25aefd5949dd" display="https://etf.dws.com//en-gb/IE000HY30YW6-s-p-500-swap-ii-ucits-etf-1c/"/>
+    <x:hyperlink ref="B59:B59" r:id="R454d9d4697684341" display="https://etf.dws.com//en-gb/IE000IDLWOL4-s-p-500-equal-weight-scored-screened-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B60:B60" r:id="R38c31b16471843e6" display="https://etf.dws.com//en-gb/IE000INYW0A7-msci-world-swap-ii-ucits-etf-1c/"/>
+    <x:hyperlink ref="B61:B61" r:id="R9acde0cadff44056" display="https://etf.dws.com//en-gb/IE000ISS8DB2-msci-world-small-cap-ucits-etf-1d/"/>
+    <x:hyperlink ref="B62:B62" r:id="R4ef3a226f6694bcf" display="https://etf.dws.com//en-gb/IE000JZYIUN0-msci-global-sdg-7-affordable-and-clean-energy-ucits-etf-1c/"/>
+    <x:hyperlink ref="B63:B63" r:id="Red6b53faeab742ab" display="https://etf.dws.com//en-gb/IE000KD0BZ68-msci-genomic-healthcare-innovation-ucits-etf-1c/"/>
+    <x:hyperlink ref="B64:B64" r:id="R740c16b0929f4244" display="https://etf.dws.com//en-gb/IE000L2IS494-msci-global-social-fairness-contributors-ucits-etf-1c/"/>
+    <x:hyperlink ref="B65:B65" r:id="Rf5e0764204f3456a" display="https://etf.dws.com//en-gb/IE000L6ZMMC4-ftse-all-world-ucits-etf-1c/"/>
+    <x:hyperlink ref="B66:B66" r:id="R7b3218fda6e748fc" display="https://etf.dws.com//en-gb/IE000LAUZQT6-msci-world-value-esg-ucits-etf-1c/"/>
+    <x:hyperlink ref="B67:B67" r:id="R8cf99e7a69424c67" display="https://etf.dws.com//en-gb/IE000LOSV2D0-usa-biodiversity-focus-sri-ucits-etf-1c/"/>
+    <x:hyperlink ref="B68:B68" r:id="R9f3347e3360343a9" display="https://etf.dws.com//en-gb/IE000M8F3JA6-global-growth-leaders-active-ucits-etf-1c/"/>
+    <x:hyperlink ref="B69:B69" r:id="R2ade6944a48f4dbe" display="https://etf.dws.com//en-gb/IE000MCVFK47-eur-corporate-green-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B70:B70" r:id="R871a40d5b9754ce1" display="https://etf.dws.com//en-gb/IE000ME8PWJ4-msci-world-utilities-ucits-etf-1d/"/>
+    <x:hyperlink ref="B71:B71" r:id="R5ba89c3bfe774ad1" display="https://etf.dws.com//en-gb/IE000MF9SZ46-msci-nordic-ucits-etf-2c-gbp-hedged/"/>
+    <x:hyperlink ref="B72:B72" r:id="Rfa4e1b8d87a34895" display="https://etf.dws.com//en-gb/IE000N5GJDD7-s-p-500-equal-weight-ucits-etf-1d-gbp-hedged/"/>
+    <x:hyperlink ref="B73:B73" r:id="R79f73d196cac4fc2" display="https://etf.dws.com//en-gb/IE000N9MLVT1-msci-europe-climate-transition-ucits-etf-1c/"/>
+    <x:hyperlink ref="B74:B74" r:id="R7ddcb2721ed74631" display="https://etf.dws.com//en-gb/IE000NS5HRY9-msci-world-high-dividend-yield-esg-ucits-etf-1d/"/>
+    <x:hyperlink ref="B75:B75" r:id="Raf6bc1166cd44568" display="https://etf.dws.com//en-gb/IE000O7Q2E56-electrification-technologies-smart-grid-ucits-etf-1c/"/>
+    <x:hyperlink ref="B76:B76" r:id="R68c3d189c2ee4c19" display="https://etf.dws.com//en-gb/IE000ONQ3X90-msci-world-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B77:B77" r:id="Rb53a08ef7803407e" display="https://etf.dws.com//en-gb/IE000P4AYI47-msci-world-climate-transition-ucits-etf-1c/"/>
+    <x:hyperlink ref="B78:B78" r:id="Red62fdeb21e6474f" display="https://etf.dws.com//en-gb/IE000PDUVTF3-msci-usa-swap-ii-ucits-etf-1c/"/>
+    <x:hyperlink ref="B79:B79" r:id="R0e37f433418d4521" display="https://etf.dws.com//en-gb/IE000PSF3A70-msci-global-sdgs-ucits-etf-1c/"/>
+    <x:hyperlink ref="B80:B80" r:id="R641b8886454a433e" display="https://etf.dws.com//en-gb/IE000QVYFUT7-india-government-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B81:B81" r:id="R59543442e8bf41f0" display="https://etf.dws.com//en-gb/IE000RNHIKK1-msci-usa-health-care-ucits-etf-1c/"/>
+    <x:hyperlink ref="B82:B82" r:id="R7aef4f6cc8114abe" display="https://etf.dws.com//en-gb/IE000SRQBBT6-s-p-500-defensive-shareholder-yield-ucits-etf-1c/"/>
+    <x:hyperlink ref="B83:B83" r:id="Read5dac7e63f4296" display="https://etf.dws.com//en-gb/IE000SZ25OI0-s-p-500-equal-weight-scored-screened-ucits-etf-4c-gbp-hedged/"/>
+    <x:hyperlink ref="B84:B84" r:id="R88b7d6f2b5744dde" display="https://etf.dws.com//en-gb/IE000TL3PL69-msci-world-momentum-esg-ucits-etf-1c/"/>
+    <x:hyperlink ref="B85:B85" r:id="R3a1f6e9debc54e1a" display="https://etf.dws.com//en-gb/IE000TSML5I8-msci-usa-screened-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B86:B86" r:id="Rd1d369c2083d4310" display="https://etf.dws.com//en-gb/IE000TZT8TI0-emerging-markets-net-zero-pathway-paris-aligned-ucits-etf-1c/"/>
+    <x:hyperlink ref="B87:B87" r:id="R5617f9754a14474a" display="https://etf.dws.com//en-gb/IE000UATQPE2-msci-world-small-cap-esg-ucits-etf-1c/"/>
+    <x:hyperlink ref="B88:B88" r:id="Rc7d90a58d8914d5c" display="https://etf.dws.com//en-gb/IE000UMV0L21-msci-usa-esg-ucits-etf-1d/"/>
+    <x:hyperlink ref="B89:B89" r:id="R47bfdac15d774fb3" display="https://etf.dws.com//en-gb/IE000UP2BIZ9-s-p-500-ucits-etf-4d/"/>
+    <x:hyperlink ref="B90:B90" r:id="R02fade0e4fb94e82" display="https://etf.dws.com//en-gb/IE000UX5WPU4-iboxx-eur-corporate-bond-yield-plus-ucits-etf-1c/"/>
+    <x:hyperlink ref="B91:B91" r:id="R4e7cda0b4dd643dc" display="https://etf.dws.com//en-gb/IE000UZCJS58-world-net-zero-pathway-paris-aligned-ucits-etf-1c/"/>
+    <x:hyperlink ref="B92:B92" r:id="R4c350814c3654eff" display="https://etf.dws.com//en-gb/IE000V04SL39-msci-usa-high-dividend-yield-esg-ucits-etf-1d/"/>
+    <x:hyperlink ref="B93:B93" r:id="R7c3705eb5cce4e3f" display="https://etf.dws.com//en-gb/IE000V0GDVU7-msci-global-sdg-11-sustainable-cities-ucits-etf-1c/"/>
+    <x:hyperlink ref="B94:B94" r:id="Rd84f4ced4587421d" display="https://etf.dws.com//en-gb/IE000VCBWFL8-msci-emu-high-dividend-yield-esg-ucits-etf-1d/"/>
+    <x:hyperlink ref="B95:B95" r:id="R9077c544ffc4463b" display="https://etf.dws.com//en-gb/IE000VCTBRW6-msci-world-industrials-ucits-etf-1d/"/>
+    <x:hyperlink ref="B96:B96" r:id="R5ac5d5c2e6af438a" display="https://etf.dws.com//en-gb/IE000VXC51U5-msci-ac-world-screened-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B97:B97" r:id="R12b653c221804d6d" display="https://etf.dws.com//en-gb/IE000W6L2AI3-msci-emu-climate-transition-ucits-etf-1c/"/>
+    <x:hyperlink ref="B98:B98" r:id="Rb7f126cce20b4735" display="https://etf.dws.com//en-gb/IE000WGF1X01-msci-ac-world-screened-ucits-etf-5c-usd-hedged/"/>
+    <x:hyperlink ref="B99:B99" r:id="R63195ac1bb154f1e" display="https://etf.dws.com//en-gb/IE000WHO5BF2-usd-high-yield-corporate-bond-screened-ucits-etf-2c-gbp-hedged/"/>
+    <x:hyperlink ref="B100:B100" r:id="R9054e703975e460c" display="https://etf.dws.com//en-gb/IE000WQ16XQ4-msci-europe-high-dividend-yield-esg-ucits-etf-1d/"/>
+    <x:hyperlink ref="B101:B101" r:id="Rf8a2fb7306644d8a" display="https://etf.dws.com//en-gb/IE000X1GW0A7-msci-world-imi-ucits-etf-1c/"/>
+    <x:hyperlink ref="B102:B102" r:id="R99349e78dd0c4561" display="https://etf.dws.com//en-gb/IE000X4A4GV2-global-equity-top-active-ucits-etf-1c/"/>
+    <x:hyperlink ref="B103:B103" r:id="R1900a1b5b56f4b80" display="https://etf.dws.com//en-gb/IE000X5MRP46-msci-usa-financials-ucits-etf-1c/"/>
+    <x:hyperlink ref="B104:B104" r:id="R257f65e2df9e4418" display="https://etf.dws.com//en-gb/IE000X63FXN4-usd-corporate-green-bond-ucits-etf-1d-gbp-hedged/"/>
+    <x:hyperlink ref="B105:B105" r:id="Rbaadeeb30a1d4c1b" display="https://etf.dws.com//en-gb/IE000X6Z71P5-msci-usa-consumer-staples-ucits-etf-1c/"/>
+    <x:hyperlink ref="B106:B106" r:id="R1dcc564a1d13482e" display="https://etf.dws.com//en-gb/IE000XOQ9TK4-msci-next-generation-internet-innovation-ucits-etf-1c/"/>
+    <x:hyperlink ref="B107:B107" r:id="R0c0a3b078258498e" display="https://etf.dws.com//en-gb/IE000Y6L6LE6-emu-net-zero-pathway-paris-aligned-ucits-etf-1c/"/>
+    <x:hyperlink ref="B108:B108" r:id="Rddc74c222cce47b3" display="https://etf.dws.com//en-gb/IE000Y6ZXZ48-msci-global-circular-economy-ucits-etf-1c/"/>
+    <x:hyperlink ref="B109:B109" r:id="Ra6f2f8ec14f448a2" display="https://etf.dws.com//en-gb/IE000YDOORK7-msci-fintech-innovation-ucits-etf-1c/"/>
+    <x:hyperlink ref="B110:B110" r:id="Rce18a657d1dd41e6" display="https://etf.dws.com//en-gb/IE000YKHGYN2-ftse-all-world-ex-us-ucits-etf-1c/"/>
+    <x:hyperlink ref="B111:B111" r:id="R9d86815c7b91441c" display="https://etf.dws.com//en-gb/IE000Z0FC0G5-msci-world-ex-usa-ucits-etf-1d/"/>
+    <x:hyperlink ref="B112:B112" r:id="Re1f7103bacbc4592" display="https://etf.dws.com//en-gb/IE000Z9SJA06-s-p-500-ucits-etf-4c/"/>
+    <x:hyperlink ref="B113:B113" r:id="Rac77a08e4a81494e" display="https://etf.dws.com//en-gb/IE00B3Y8D011-portfolio-income-ucits-etf-1d/"/>
+    <x:hyperlink ref="B114:B114" r:id="R4eb661b587704d10" display="https://etf.dws.com//en-gb/IE00B8KMSQ34-s-p-500-ucits-etf-3c-chf-hedged/"/>
+    <x:hyperlink ref="B115:B115" r:id="R7d9353edcf84427d" display="https://etf.dws.com//en-gb/IE00B9MRHC27-msci-nordic-ucits-etf-1d/"/>
+    <x:hyperlink ref="B116:B116" r:id="R626094e05bb34816" display="https://etf.dws.com//en-gb/IE00B9MRJJ36-mdax-esg-screened-ucits-etf-1d/"/>
+    <x:hyperlink ref="B117:B117" r:id="Rc7a744f7d773441b" display="https://etf.dws.com//en-gb/IE00BCHWNQ94-msci-world-screened-ucits-etf-1d/"/>
+    <x:hyperlink ref="B118:B118" r:id="R6e0cbc1b58004bd1" display="https://etf.dws.com//en-gb/IE00BCHWNS19-msci-usa-energy-ucits-etf-1d/"/>
+    <x:hyperlink ref="B119:B119" r:id="R01e315c08e0546ec" display="https://etf.dws.com//en-gb/IE00BCHWNT26-msci-usa-financials-ucits-etf-1d/"/>
+    <x:hyperlink ref="B120:B120" r:id="R4a95cf5c08ba4b85" display="https://etf.dws.com//en-gb/IE00BCHWNV48-msci-usa-industrials-ucits-etf-1d/"/>
+    <x:hyperlink ref="B121:B121" r:id="Re15e710312e3465f" display="https://etf.dws.com//en-gb/IE00BCHWNW54-msci-usa-health-care-ucits-etf-1d/"/>
+    <x:hyperlink ref="B122:B122" r:id="Rab4273f511e14e43" display="https://etf.dws.com//en-gb/IE00BD4DX952-esg-usd-emerging-markets-bond-quality-weighted-ucits-etf-1d/"/>
+    <x:hyperlink ref="B123:B123" r:id="Rd5f5498f0be54525" display="https://etf.dws.com//en-gb/IE00BD4DXB77-esg-usd-emerging-markets-bond-quality-weighted-ucits-etf-2d-eur-hedged/"/>
+    <x:hyperlink ref="B124:B124" r:id="Rbc570920a61c42b3" display="https://etf.dws.com//en-gb/IE00BDB7J586-msci-usa-minimum-volatility-ucits-etf-1d/"/>
+    <x:hyperlink ref="B125:B125" r:id="R7ac47e8f48e04f0b" display="https://etf.dws.com//en-gb/IE00BDGN9Z19-msci-emu-screened-ucits-etf-1d/"/>
+    <x:hyperlink ref="B126:B126" r:id="Rc768a50e2fd547d6" display="https://etf.dws.com//en-gb/IE00BDR5HM97-usd-high-yield-corporate-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B127:B127" r:id="R3d42717da8cb4999" display="https://etf.dws.com//en-gb/IE00BDR5HN05-usd-high-yield-corporate-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B128:B128" r:id="Rd8d8356b9aae465e" display="https://etf.dws.com//en-gb/IE00BDVPTJ63-msci-usa-banks-ucits-etf-1d/"/>
+    <x:hyperlink ref="B129:B129" r:id="Rb726b9f9eead4a10" display="https://etf.dws.com//en-gb/IE00BF8J5974-usd-corporate-bond-short-duration-sri-pab-ucits-etf-1d/"/>
+    <x:hyperlink ref="B130:B130" r:id="R7d33f4cd94304aca" display="https://etf.dws.com//en-gb/IE00BFMKQ930-usd-corporate-bond-short-duration-sri-pab-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B131:B131" r:id="R4f68f7509eae4600" display="https://etf.dws.com//en-gb/IE00BFMKQC67-usd-corporate-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B132:B132" r:id="R9e6403740cd146a9" display="https://etf.dws.com//en-gb/IE00BFMNHK08-msci-europe-esg-ucits-etf-1c/"/>
+    <x:hyperlink ref="B133:B133" r:id="R93b176ab89674a29" display="https://etf.dws.com//en-gb/IE00BFMNPS42-msci-usa-esg-ucits-etf-1c/"/>
+    <x:hyperlink ref="B134:B134" r:id="R360ad492fdb54e8f" display="https://etf.dws.com//en-gb/IE00BG04LT92-usd-high-yield-corporate-bond-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B135:B135" r:id="Rd5918fd2d0c8465a" display="https://etf.dws.com//en-gb/IE00BG04LV15-usd-high-yield-corporate-bond-ucits-etf-4d-gbp-hedged/"/>
+    <x:hyperlink ref="B136:B136" r:id="Rfefa61ccc4654076" display="https://etf.dws.com//en-gb/IE00BG04LY46-usd-corporate-bond-ucits-etf-5d-gbp-hedged/"/>
+    <x:hyperlink ref="B137:B137" r:id="Reeff7d7972c840f3" display="https://etf.dws.com//en-gb/IE00BG04LZ52-msci-usa-ucits-etf-3c-chf-hedged/"/>
+    <x:hyperlink ref="B138:B138" r:id="R8cba555303ae46a4" display="https://etf.dws.com//en-gb/IE00BG04M077-msci-usa-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B139:B139" r:id="R22f0f3f4dbca45ee" display="https://etf.dws.com//en-gb/IE00BG36TC12-msci-japan-esg-ucits-etf-1c/"/>
+    <x:hyperlink ref="B140:B140" r:id="Rd8d59a4424c14a9b" display="https://etf.dws.com//en-gb/IE00BG370F43-msci-emerging-markets-esg-ucits-etf-1c/"/>
+    <x:hyperlink ref="B141:B141" r:id="R79894e4b7c864e3f" display="https://etf.dws.com//en-gb/IE00BGHQ0G80-msci-ac-world-screened-ucits-etf-1c/"/>
+    <x:hyperlink ref="B142:B142" r:id="R6d61c5c17cfd40d1" display="https://etf.dws.com//en-gb/IE00BGJWX091-s-p-500-ucits-etf-1d-eur-hedged/"/>
+    <x:hyperlink ref="B143:B143" r:id="R968755d179624efd" display="https://etf.dws.com//en-gb/IE00BGQYRQ28-msci-usa-consumer-staples-ucits-etf-1d/"/>
+    <x:hyperlink ref="B144:B144" r:id="R7165d240ed224892" display="https://etf.dws.com//en-gb/IE00BGQYRR35-msci-usa-consumer-discretionary-ucits-etf-1d/"/>
+    <x:hyperlink ref="B145:B145" r:id="Ra4cd7963da644bb0" display="https://etf.dws.com//en-gb/IE00BGQYRS42-msci-usa-information-technology-ucits-etf-1d/"/>
+    <x:hyperlink ref="B146:B146" r:id="R7d2d7512d07f4f04" display="https://etf.dws.com//en-gb/IE00BGV5VM45-s-p-europe-ex-uk-ucits-etf-1d/"/>
+    <x:hyperlink ref="B147:B147" r:id="R4cd22bcb61934e6e" display="https://etf.dws.com//en-gb/IE00BGV5VN51-artificial-intelligence-big-data-ucits-etf-1c/"/>
+    <x:hyperlink ref="B148:B148" r:id="Rf7f22fc2754341ea" display="https://etf.dws.com//en-gb/IE00BGV5VR99-future-mobility-ucits-etf-1c/"/>
+    <x:hyperlink ref="B149:B149" r:id="Reb885d1aa62140a2" display="https://etf.dws.com//en-gb/IE00BH361H73-msci-north-america-high-dividend-yield-ucits-etf-1c/"/>
+    <x:hyperlink ref="B150:B150" r:id="R316862a75e6e4102" display="https://etf.dws.com//en-gb/IE00BJ0KDQ92-msci-world-ucits-etf-1c/"/>
+    <x:hyperlink ref="B151:B151" r:id="Ra0f49cd1f2934e74" display="https://etf.dws.com//en-gb/IE00BJ0KDR00-msci-usa-ucits-etf-1c/"/>
+    <x:hyperlink ref="B152:B152" r:id="R2ac38bcda42c4322" display="https://etf.dws.com//en-gb/IE00BJZ2DC62-msci-usa-screened-ucits-etf-1c/"/>
+    <x:hyperlink ref="B153:B153" r:id="R8e85655727a749d8" display="https://etf.dws.com//en-gb/IE00BJZ2DD79-russell-2000-ucits-etf-1c/"/>
+    <x:hyperlink ref="B154:B154" r:id="R7f4d821b5f164b26" display="https://etf.dws.com//en-gb/IE00BK1PV445-msci-usa-ucits-etf-1d/"/>
+    <x:hyperlink ref="B155:B155" r:id="R3e863313fb3f4ce6" display="https://etf.dws.com//en-gb/IE00BK1PV551-msci-world-ucits-etf-1d/"/>
+    <x:hyperlink ref="B156:B156" r:id="R99bb1f31a5ff405a" display="https://etf.dws.com//en-gb/IE00BL25JL35-msci-world-quality-ucits-etf-1c/"/>
+    <x:hyperlink ref="B157:B157" r:id="R1dd6957bb35948a9" display="https://etf.dws.com//en-gb/IE00BL25JM42-msci-world-value-ucits-etf-1c/"/>
+    <x:hyperlink ref="B158:B158" r:id="R10fe2c7034884500" display="https://etf.dws.com//en-gb/IE00BL25JN58-msci-world-minimum-volatility-ucits-etf-1c/"/>
+    <x:hyperlink ref="B159:B159" r:id="R31f61f7b43414af5" display="https://etf.dws.com//en-gb/IE00BL25JP72-msci-world-momentum-ucits-etf-1c/"/>
+    <x:hyperlink ref="B160:B160" r:id="Rb9e21078163442c0" display="https://etf.dws.com//en-gb/IE00BL58LJ19-usd-corporate-bond-sri-pab-ucits-etf-1c/"/>
+    <x:hyperlink ref="B161:B161" r:id="Re7af6d0f5a2f46dc" display="https://etf.dws.com//en-gb/IE00BL58LL31-usd-corporate-bond-sri-pab-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B162:B162" r:id="R5a5ded62d3ed45df" display="https://etf.dws.com//en-gb/IE00BLNMYC90-s-p-500-equal-weight-ucits-etf-1c/"/>
+    <x:hyperlink ref="B163:B163" r:id="Re3512e8a0a3a4706" display="https://etf.dws.com//en-gb/IE00BM67HJ62-msci-emerging-markets-ex-china-ucits-etf-1c/"/>
+    <x:hyperlink ref="B164:B164" r:id="Rfb185c1cc84741cc" display="https://etf.dws.com//en-gb/IE00BM67HK77-msci-world-health-care-ucits-etf-1c/"/>
+    <x:hyperlink ref="B165:B165" r:id="R275229fd4a004e1b" display="https://etf.dws.com//en-gb/IE00BM67HL84-msci-world-financials-ucits-etf-1c/"/>
+    <x:hyperlink ref="B166:B166" r:id="Rd83376d1533b41ea" display="https://etf.dws.com//en-gb/IE00BM67HM91-msci-world-energy-ucits-etf-1c/"/>
+    <x:hyperlink ref="B167:B167" r:id="R307c52f5f22a4da2" display="https://etf.dws.com//en-gb/IE00BM67HN09-msci-world-consumer-staples-ucits-etf-1c/"/>
+    <x:hyperlink ref="B168:B168" r:id="Rf2d384549d7f442c" display="https://etf.dws.com//en-gb/IE00BM67HP23-msci-world-consumer-discretionary-ucits-etf-1c/"/>
+    <x:hyperlink ref="B169:B169" r:id="R60e39ffff20b4e4a" display="https://etf.dws.com//en-gb/IE00BM67HQ30-msci-world-utilities-ucits-etf-1c/"/>
+    <x:hyperlink ref="B170:B170" r:id="Ra1999e719dde4409" display="https://etf.dws.com//en-gb/IE00BM67HR47-msci-world-communication-services-ucits-etf-1c/"/>
+    <x:hyperlink ref="B171:B171" r:id="R34a64472d6424420" display="https://etf.dws.com//en-gb/IE00BM67HS53-msci-world-materials-ucits-etf-1c/"/>
+    <x:hyperlink ref="B172:B172" r:id="R34f48a0284fe41ab" display="https://etf.dws.com//en-gb/IE00BM67HT60-msci-world-information-technology-ucits-etf-1c/"/>
+    <x:hyperlink ref="B173:B173" r:id="Rd78cbd5755274dec" display="https://etf.dws.com//en-gb/IE00BM67HV82-msci-world-industrials-ucits-etf-1c/"/>
+    <x:hyperlink ref="B174:B174" r:id="R61cc8912479a4536" display="https://etf.dws.com//en-gb/IE00BM67HW99-s-p-500-ucits-etf-1c-eur-hedged/"/>
+    <x:hyperlink ref="B175:B175" r:id="Rb828f95c0cb04777" display="https://etf.dws.com//en-gb/IE00BM67HX07-s-p-500-ucits-etf-2c-gbp-hedged/"/>
+    <x:hyperlink ref="B176:B176" r:id="R1d58c792a088431c" display="https://etf.dws.com//en-gb/IE00BM97MR69-us-treasuries-ultrashort-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B177:B177" r:id="R53ca6e2fc4d94201" display="https://etf.dws.com//en-gb/IE00BM97MV06-us-treasuries-ultrashort-bond-ucits-etf-3c-mxn-hedged/"/>
+    <x:hyperlink ref="B178:B178" r:id="R6eea608bd1434e92" display="https://etf.dws.com//en-gb/IE00BMCFJ320-usd-corporate-bond-ucits-etf-6c-mxn-hedged/"/>
+    <x:hyperlink ref="B179:B179" r:id="Re67161dd024a4b86" display="https://etf.dws.com//en-gb/IE00BMFKG444-nasdaq-100-ucits-etf-1c/"/>
+    <x:hyperlink ref="B180:B180" r:id="Re10d1ea436c54497" display="https://etf.dws.com//en-gb/IE00BMY76136-msci-world-esg-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B181:B181" r:id="Rbeb468efb2384a79" display="https://etf.dws.com//en-gb/IE00BN2BCY94-developed-green-real-estate-esg-ucits-etf-1c/"/>
+    <x:hyperlink ref="B182:B182" r:id="R1c06277083c8409f" display="https://etf.dws.com//en-gb/IE00BNC1G699-msci-emu-esg-ucits-etf-1c/"/>
+    <x:hyperlink ref="B183:B183" r:id="R4540bf7b9a6044be" display="https://etf.dws.com//en-gb/IE00BNC1G707-msci-usa-communication-services-ucits-etf-1d/"/>
+    <x:hyperlink ref="B184:B184" r:id="R91783c06942c4241" display="https://etf.dws.com//en-gb/IE00BNKF6C99-stoxx-european-market-leaders-ucits-etf-1c/"/>
+    <x:hyperlink ref="B185:B185" r:id="R0e99e12c540548ce" display="https://etf.dws.com//en-gb/IE00BP8FKB21-ftse-developed-europe-ex-uk-real-estate-ucits-etf-1c/"/>
+    <x:hyperlink ref="B186:B186" r:id="Reae11e181ada4f22" display="https://etf.dws.com//en-gb/IE00BPVLQD13-msci-japan-screened-ucits-etf-1d/"/>
+    <x:hyperlink ref="B187:B187" r:id="Re0bd606d79004d3f" display="https://etf.dws.com//en-gb/IE00BPVLQF37-msci-japan-screened-ucits-etf-2d-gbp-hedged/"/>
+    <x:hyperlink ref="B188:B188" r:id="Rf30ba0ddb5e74ba3" display="https://etf.dws.com//en-gb/IE00BQXKVQ19-msci-gcc-select-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B189:B189" r:id="R3c9fac7d8ff54e63" display="https://etf.dws.com//en-gb/IE00BRB36B93-msci-japan-screened-ucits-etf-3c-eur-hedged/"/>
+    <x:hyperlink ref="B190:B190" r:id="R1bc5d891af484c91" display="https://etf.dws.com//en-gb/IE00BTGD1B38-msci-japan-screened-ucits-etf-4c-usd-hedged/"/>
+    <x:hyperlink ref="B191:B191" r:id="R07652426e7974c52" display="https://etf.dws.com//en-gb/IE00BTJRMP35-msci-emerging-markets-ucits-etf-1c/"/>
+    <x:hyperlink ref="B192:B192" r:id="R8ab8cdf09d944b31" display="https://etf.dws.com//en-gb/IE00BYPHT736-iboxx-eur-corporate-bond-yield-plus-ucits-etf-1d/"/>
+    <x:hyperlink ref="B193:B193" r:id="R57b7aef52dd948b2" display="https://etf.dws.com//en-gb/IE00BYZNF849-global-infrastructure-esg-ucits-etf-1c/"/>
+    <x:hyperlink ref="B194:B194" r:id="R9bdfda577447441d" display="https://etf.dws.com//en-gb/IE00BZ02LR44-msci-world-esg-ucits-etf-1c/"/>
+    <x:hyperlink ref="B195:B195" r:id="Rebe420a315cd406b" display="https://etf.dws.com//en-gb/IE00BZ036H21-usd-corporate-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B196:B196" r:id="R8165bfb75f074f39" display="https://etf.dws.com//en-gb/IE00BZ036J45-usd-corporate-bond-ucits-etf-2d-eur-hedged/"/>
+    <x:hyperlink ref="B197:B197" r:id="R96bb8896595a45a0" display="https://etf.dws.com//en-gb/IE00BZ1BS790-msci-world-ucits-etf-2d-gbp-hedged/"/>
+    <x:hyperlink ref="B198:B198" r:id="R557d9360ec7245dd" display="https://etf.dws.com//en-gb/LU0274208692-msci-world-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B199:B199" r:id="R3368c572c9d84bb6" display="https://etf.dws.com//en-gb/LU0274209237-msci-europe-ucits-etf-1c/"/>
+    <x:hyperlink ref="B200:B200" r:id="Ra17032a1bc0d408b" display="https://etf.dws.com//en-gb/LU0274209740-msci-japan-ucits-etf-1c/"/>
+    <x:hyperlink ref="B201:B201" r:id="R4d8810ab781441e1" display="https://etf.dws.com//en-gb/LU0274210672-msci-usa-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B202:B202" r:id="R806a79290ca24e1c" display="https://etf.dws.com//en-gb/LU0274211217-euro-stoxx-50-ucits-etf-1d/"/>
+    <x:hyperlink ref="B203:B203" r:id="R32ff1a011a014d6c" display="https://etf.dws.com//en-gb/LU0274211480-dax-ucits-etf-1c/"/>
+    <x:hyperlink ref="B204:B204" r:id="R3b466af3391a45ea" display="https://etf.dws.com//en-gb/LU0274212538-ftse-mib-ucits-etf-1d/"/>
+    <x:hyperlink ref="B205:B205" r:id="Rfdd5d6fd2dc644ba" display="https://etf.dws.com//en-gb/LU0274221281-switzerland-ucits-etf-1d/"/>
+    <x:hyperlink ref="B206:B206" r:id="R582b56275df64b89" display="https://etf.dws.com//en-gb/LU0290355717-eurozone-government-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B207:B207" r:id="R456ab742167744e6" display="https://etf.dws.com//en-gb/LU0290356871-eurozone-government-bond-1-3-ucits-etf-1c/"/>
+    <x:hyperlink ref="B208:B208" r:id="R01456749f3874852" display="https://etf.dws.com//en-gb/LU0290356954-eurozone-government-bond-3-5-ucits-etf-1c/"/>
+    <x:hyperlink ref="B209:B209" r:id="R1688b3f3a9f34f87" display="https://etf.dws.com//en-gb/LU0290357176-eurozone-government-bond-5-7-ucits-etf-1c/"/>
+    <x:hyperlink ref="B210:B210" r:id="R22a1147acd0640e0" display="https://etf.dws.com//en-gb/LU0290357259-eurozone-government-bond-7-10-ucits-etf-1c/"/>
+    <x:hyperlink ref="B211:B211" r:id="Rb7b7f73b94614318" display="https://etf.dws.com//en-gb/LU0290357507-eurozone-government-bond-15-30-ucits-etf-1c/"/>
+    <x:hyperlink ref="B212:B212" r:id="Rb0621293b6be48e6" display="https://etf.dws.com//en-gb/LU0290357846-eurozone-government-bond-25-ucits-etf-1c/"/>
+    <x:hyperlink ref="B213:B213" r:id="Rc8ca2e3a183c40b4" display="https://etf.dws.com//en-gb/LU0290357929-global-inflation-linked-bond-ucits-etf-1c-eur-hedged/"/>
+    <x:hyperlink ref="B214:B214" r:id="Ree1dd9dbbee240e1" display="https://etf.dws.com//en-gb/LU0290358224-eurozone-inflation-linked-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B215:B215" r:id="R170d33f715ad45bd" display="https://etf.dws.com//en-gb/LU0290358497-eur-overnight-rate-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B216:B216" r:id="R68ad86136931401f" display="https://etf.dws.com//en-gb/LU0292095535-euro-stoxx-quality-dividend-ucits-etf-1d/"/>
+    <x:hyperlink ref="B217:B217" r:id="Rc3189d070daa4ab2" display="https://etf.dws.com//en-gb/LU0292096186-stoxx-global-select-dividend-100-swap-ucits-etf-1d/"/>
+    <x:hyperlink ref="B218:B218" r:id="Rdd83f49fbe164dad" display="https://etf.dws.com//en-gb/LU0292097234-ftse-100-income-ucits-etf-1d/"/>
+    <x:hyperlink ref="B219:B219" r:id="R88bdedd2d0d14f94" display="https://etf.dws.com//en-gb/LU0292097317-ftse-250-ucits-etf-1d/"/>
+    <x:hyperlink ref="B220:B220" r:id="R9cfe42cecfb34486" display="https://etf.dws.com//en-gb/LU0292097747-msci-uk-esg-ucits-etf-1d/"/>
+    <x:hyperlink ref="B221:B221" r:id="Ra479fd931c864320" display="https://etf.dws.com//en-gb/LU0292100046-msci-korea-ucits-etf-1c/"/>
+    <x:hyperlink ref="B222:B222" r:id="R3d41be5e11b042ee" display="https://etf.dws.com//en-gb/LU0292100806-msci-europe-materials-ucits-etf-1c/"/>
+    <x:hyperlink ref="B223:B223" r:id="R75dbfd22494b44e2" display="https://etf.dws.com//en-gb/LU0292103222-msci-europe-health-care-ucits-etf-1c/"/>
+    <x:hyperlink ref="B224:B224" r:id="R2d69efddbead4d70" display="https://etf.dws.com//en-gb/LU0292103651-msci-europe-financials-ucits-etf-1c/"/>
+    <x:hyperlink ref="B225:B225" r:id="R8e9465806541466a" display="https://etf.dws.com//en-gb/LU0292104030-msci-europe-communication-services-ucits-etf-1c/"/>
+    <x:hyperlink ref="B226:B226" r:id="R2a1cc0637b584c82" display="https://etf.dws.com//en-gb/LU0292104469-msci-europe-information-technology-ucits-etf-1c/"/>
+    <x:hyperlink ref="B227:B227" r:id="R6e70c425140846c0" display="https://etf.dws.com//en-gb/LU0292104899-msci-europe-utilities-ucits-etf-1c/"/>
+    <x:hyperlink ref="B228:B228" r:id="Ra40e1b5fcde548b7" display="https://etf.dws.com//en-gb/LU0292105359-msci-europe-consumer-staples-ucits-etf-1c/"/>
+    <x:hyperlink ref="B229:B229" r:id="Rc17414a758db4813" display="https://etf.dws.com//en-gb/LU0292106084-msci-europe-industrials-ucits-etf-1c/"/>
+    <x:hyperlink ref="B230:B230" r:id="Ra2120980c51e443b" display="https://etf.dws.com//en-gb/LU0292106167-bloomberg-commodity-ex-agriculture-livestock-swap-ucits-etf-1c-eur-hedged/"/>
+    <x:hyperlink ref="B231:B231" r:id="Rcc4eb6b835764c74" display="https://etf.dws.com//en-gb/LU0292106241-shortdax-daily-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B232:B232" r:id="R86ed63b971c04672" display="https://etf.dws.com//en-gb/LU0292106753-euro-stoxx-50-short-daily-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B233:B233" r:id="Rd4b3c70b7fb649eb" display="https://etf.dws.com//en-gb/LU0292107645-msci-emerging-markets-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B234:B234" r:id="R86543ab740a4499e" display="https://etf.dws.com//en-gb/LU0292107991-msci-em-asia-screened-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B235:B235" r:id="R7eae808f2342448b" display="https://etf.dws.com//en-gb/LU0292108619-msci-em-latin-america-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B236:B236" r:id="R652de2a196194000" display="https://etf.dws.com//en-gb/LU0292109005-msci-em-europe-middle-east-africa-esg-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B237:B237" r:id="R767cc72e141c4548" display="https://etf.dws.com//en-gb/LU0292109187-msci-taiwan-ucits-etf-1c/"/>
+    <x:hyperlink ref="B238:B238" r:id="Rd427911383834af2" display="https://etf.dws.com//en-gb/LU0292109344-msci-brazil-ucits-etf-1c/"/>
+    <x:hyperlink ref="B239:B239" r:id="R45cd9dcad9ba4c75" display="https://etf.dws.com//en-gb/LU0292109690-nifty-50-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B240:B240" r:id="Rc6ce4b4fabb6488d" display="https://etf.dws.com//en-gb/LU0292109856-msci-china-a-ucits-etf-1c/"/>
+    <x:hyperlink ref="B241:B241" r:id="R8ab853abc6b74961" display="https://etf.dws.com//en-gb/LU0321462870-itraxx-crossover-short-daily-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B242:B242" r:id="R74be5883cfb44e4d" display="https://etf.dws.com//en-gb/LU0321462953-j-p-morgan-usd-emerging-markets-bond-ucits-etf-1c-eur-hedged/"/>
+    <x:hyperlink ref="B243:B243" r:id="Rb89cc1d835844860" display="https://etf.dws.com//en-gb/LU0321464652-gbp-overnight-rate-swap-ucits-etf-1d/"/>
+    <x:hyperlink ref="B244:B244" r:id="R2eede0f795844475" display="https://etf.dws.com//en-gb/LU0321465469-usd-overnight-rate-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B245:B245" r:id="R78bbe03490f34142" display="https://etf.dws.com//en-gb/LU0322248146-sli-ucits-etf-1d/"/>
+    <x:hyperlink ref="B246:B246" r:id="Rb692840851444a70" display="https://etf.dws.com//en-gb/LU0322250712-lpx-private-equity-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B247:B247" r:id="R1c311ecd0e744c2c" display="https://etf.dws.com//en-gb/LU0322250985-cac-40-ucits-etf-1d/"/>
+    <x:hyperlink ref="B248:B248" r:id="R4e7584024fd44e3b" display="https://etf.dws.com//en-gb/LU0322251520-s-p-500-inverse-daily-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B249:B249" r:id="Reb817f5d4083454e" display="https://etf.dws.com//en-gb/LU0322252171-msci-ac-asia-ex-japan-esg-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B250:B250" r:id="Ra660e1b7f5f94b87" display="https://etf.dws.com//en-gb/LU0322252338-msci-pacific-ex-japan-ucits-etf-1c/"/>
+    <x:hyperlink ref="B251:B251" r:id="R0b068ee82ac34ceb" display="https://etf.dws.com//en-gb/LU0322252924-vietnam-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B252:B252" r:id="Rae8e8611d2694a82" display="https://etf.dws.com//en-gb/LU0322253229-s-p-global-infrastructure-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B253:B253" r:id="R401314b47b9949a7" display="https://etf.dws.com//en-gb/LU0322253732-msci-europe-screened-ucits-etf-1c/"/>
+    <x:hyperlink ref="B254:B254" r:id="R71007990e91e4275" display="https://etf.dws.com//en-gb/LU0322253906-msci-europe-small-cap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B255:B255" r:id="R86d138f830014c49" display="https://etf.dws.com//en-gb/LU0328473581-ftse-100-short-daily-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B256:B256" r:id="Rbb4abfe0bfd84179" display="https://etf.dws.com//en-gb/LU0328474803-s-p-asx-200-ucits-etf-1d/"/>
+    <x:hyperlink ref="B257:B257" r:id="Rce9cf32e1ecb4140" display="https://etf.dws.com//en-gb/LU0328475792-stoxx-europe-600-ucits-etf-1c/"/>
+    <x:hyperlink ref="B258:B258" r:id="R05de88c2a3574d00" display="https://etf.dws.com//en-gb/LU0328476410-s-p-select-frontier-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B259:B259" r:id="R86ec6e583c45487d" display="https://etf.dws.com//en-gb/LU0335044896-eur-overnight-rate-swap-ucits-etf-1d/"/>
+    <x:hyperlink ref="B260:B260" r:id="Rb2677653512b4a89" display="https://etf.dws.com//en-gb/LU0378818131-global-government-bond-ucits-etf-1c-eur-hedged/"/>
+    <x:hyperlink ref="B261:B261" r:id="R74f8ba7582334b28" display="https://etf.dws.com//en-gb/LU0378818560-singapore-government-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B262:B262" r:id="R372fd7a644b24a99" display="https://etf.dws.com//en-gb/LU0380865021-euro-stoxx-50-ucits-etf-1c/"/>
+    <x:hyperlink ref="B263:B263" r:id="R29137b36d0b24f81" display="https://etf.dws.com//en-gb/LU0397221945-portfolio-ucits-etf-1c/"/>
+    <x:hyperlink ref="B264:B264" r:id="R2f2dde4d263c4da2" display="https://etf.dws.com//en-gb/LU0411075020-shortdax-x2-daily-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B265:B265" r:id="R2e4edcdd69b545f5" display="https://etf.dws.com//en-gb/LU0411075376-levdax-daily-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B266:B266" r:id="R3a553aa044a049f2" display="https://etf.dws.com//en-gb/LU0411078552-s-p-500-2x-leveraged-daily-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B267:B267" r:id="R1916620777b64389" display="https://etf.dws.com//en-gb/LU0411078636-s-p-500-2x-inverse-daily-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B268:B268" r:id="R233e6d87bc4e4bdc" display="https://etf.dws.com//en-gb/LU0429458895-us-treasuries-1-3-ucits-etf-1d/"/>
+    <x:hyperlink ref="B269:B269" r:id="Re7a15fedd01f4f04" display="https://etf.dws.com//en-gb/LU0429459356-us-treasuries-ucits-etf-1d/"/>
+    <x:hyperlink ref="B270:B270" r:id="Re5d4b57dab6d440d" display="https://etf.dws.com//en-gb/LU0429790743-bloomberg-commodity-swap-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B271:B271" r:id="Ra06999b14eb94997" display="https://etf.dws.com//en-gb/LU0460391732-bloomberg-commodity-ex-agriculture-livestock-swap-ucits-etf-2c/"/>
+    <x:hyperlink ref="B272:B272" r:id="R45588d94a6764642" display="https://etf.dws.com//en-gb/LU0460391906-bloomberg-commodity-ex-agriculture-livestock-swap-ucits-etf-3c-gbp-hedged/"/>
+    <x:hyperlink ref="B273:B273" r:id="R9ceafbe8573b4aa2" display="https://etf.dws.com//en-gb/LU0468896575-germany-government-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B274:B274" r:id="Re4a7a9cbd9544e29" display="https://etf.dws.com//en-gb/LU0468897110-germany-government-bond-1-3-ucits-etf-1d/"/>
+    <x:hyperlink ref="B275:B275" r:id="Rcb09b12135034d2c" display="https://etf.dws.com//en-gb/LU0476289466-msci-mexico-ucits-etf-1c/"/>
+    <x:hyperlink ref="B276:B276" r:id="Rbc6073ac5780453b" display="https://etf.dws.com//en-gb/LU0476289540-msci-canada-screened-ucits-etf-1c/"/>
+    <x:hyperlink ref="B277:B277" r:id="Rf178963e14474760" display="https://etf.dws.com//en-gb/LU0476289623-msci-indonesia-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B278:B278" r:id="Rcae8ff3337aa41d1" display="https://etf.dws.com//en-gb/LU0478205379-eur-corporate-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B279:B279" r:id="Rc138f92ebfc4492e" display="https://etf.dws.com//en-gb/LU0478205965-eur-corporate-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B280:B280" r:id="R375443e281ce4632" display="https://etf.dws.com//en-gb/LU0484968812-eur-corporate-bond-sri-pab-ucits-etf-1d/"/>
+    <x:hyperlink ref="B281:B281" r:id="Ra1b3dd2e374e424a" display="https://etf.dws.com//en-gb/LU0484968903-eur-corporate-bond-sri-pab-ucits-etf-1c/"/>
+    <x:hyperlink ref="B282:B282" r:id="R5f6dd8eaafc14ef2" display="https://etf.dws.com//en-gb/LU0484969463-target-maturity-sept-2029-italy-and-spain-government-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B283:B283" r:id="R3e82ab8d8014449d" display="https://etf.dws.com//en-gb/LU0486851024-msci-europe-value-ucits-etf-1c/"/>
+    <x:hyperlink ref="B284:B284" r:id="Rcf9347c07509451a" display="https://etf.dws.com//en-gb/LU0489337690-ftse-developed-europe-real-estate-ucits-etf-1c/"/>
+    <x:hyperlink ref="B285:B285" r:id="Rb773908dfd3e4dc1" display="https://etf.dws.com//en-gb/LU0490618542-s-p-500-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B286:B286" r:id="Rdb2df13028f649c4" display="https://etf.dws.com//en-gb/LU0494592974-australia-government-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B287:B287" r:id="Rf95338d4c71a4ee2" display="https://etf.dws.com//en-gb/LU0514694370-msci-malaysia-ucits-etf-1c/"/>
+    <x:hyperlink ref="B288:B288" r:id="R064ba4bd09684dcb" display="https://etf.dws.com//en-gb/LU0514694701-msci-thailand-ucits-etf-1c/"/>
+    <x:hyperlink ref="B289:B289" r:id="R0b03cfeb73724905" display="https://etf.dws.com//en-gb/LU0514695187-msci-india-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B290:B290" r:id="R3b489218360547ab" display="https://etf.dws.com//en-gb/LU0514695690-msci-china-ucits-etf-1c/"/>
+    <x:hyperlink ref="B291:B291" r:id="R93a88b70d36542de" display="https://etf.dws.com//en-gb/LU0524480265-iboxx-eurozone-government-bond-yield-plus-ucits-etf-1c/"/>
+    <x:hyperlink ref="B292:B292" r:id="R9f9c8e0351284f16" display="https://etf.dws.com//en-gb/LU0592215403-msci-philippines-ucits-etf-1c/"/>
+    <x:hyperlink ref="B293:B293" r:id="Rf0788c5ec45641db" display="https://etf.dws.com//en-gb/LU0592216393-spain-ucits-etf-1c/"/>
+    <x:hyperlink ref="B294:B294" r:id="Rce91150b523544c4" display="https://etf.dws.com//en-gb/LU0592217524-msci-africa-top-50-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B295:B295" r:id="Rb02fcdeb0f334560" display="https://etf.dws.com//en-gb/LU0613540268-italy-government-bond-0-1-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B296:B296" r:id="R1868094d556048ce" display="https://etf.dws.com//en-gb/LU0614173549-eurozone-government-bond-1-3-ucits-etf-1d/"/>
+    <x:hyperlink ref="B297:B297" r:id="R682bebef72aa464d" display="https://etf.dws.com//en-gb/LU0614173895-eurozone-government-bond-3-5-ucits-etf-1d/"/>
+    <x:hyperlink ref="B298:B298" r:id="R82a673323a0f4755" display="https://etf.dws.com//en-gb/LU0641006290-global-government-bond-ucits-etf-2d-gbp-hedged/"/>
+    <x:hyperlink ref="B299:B299" r:id="Ra7aa41bd33ce472e" display="https://etf.dws.com//en-gb/LU0641006456-global-government-bond-ucits-etf-3c-usd-hedged/"/>
+    <x:hyperlink ref="B300:B300" r:id="R3d1e3daf05fb4e25" display="https://etf.dws.com//en-gb/LU0641006613-global-government-bond-ucits-etf-4c-chf-hedged/"/>
+    <x:hyperlink ref="B301:B301" r:id="R3aaf9a7dd1294467" display="https://etf.dws.com//en-gb/LU0641007009-global-inflation-linked-bond-ucits-etf-2c-usd-hedged/"/>
+    <x:hyperlink ref="B302:B302" r:id="R44f7fa8c8930443f" display="https://etf.dws.com//en-gb/LU0641007264-global-inflation-linked-bond-ucits-etf-3d-gbp-hedged/"/>
+    <x:hyperlink ref="B303:B303" r:id="Rb23e9f8b6feb4903" display="https://etf.dws.com//en-gb/LU0641007421-global-inflation-linked-bond-ucits-etf-4d-chf-hedged/"/>
+    <x:hyperlink ref="B304:B304" r:id="R27b822b42b984d46" display="https://etf.dws.com//en-gb/LU0643975161-germany-government-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B305:B305" r:id="R6851a48daffc42e4" display="https://etf.dws.com//en-gb/LU0643975591-eurozone-government-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B306:B306" r:id="R43339fb91ae44452" display="https://etf.dws.com//en-gb/LU0659578842-msci-singapore-ucits-etf-1c/"/>
+    <x:hyperlink ref="B307:B307" r:id="R4da3367999ca41a0" display="https://etf.dws.com//en-gb/LU0659579063-atx-ucits-etf-1c/"/>
+    <x:hyperlink ref="B308:B308" r:id="R01f05383e48e4e1c" display="https://etf.dws.com//en-gb/LU0659579147-msci-pakistan-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B309:B309" r:id="R4d01aa9fc01a4f70" display="https://etf.dws.com//en-gb/LU0659579733-msci-world-swap-ucits-etf-4c-eur-hedged/"/>
+    <x:hyperlink ref="B310:B310" r:id="R2fd58fc2e1654eb4" display="https://etf.dws.com//en-gb/LU0659580079-msci-japan-ucits-etf-4c-eur-hedged/"/>
+    <x:hyperlink ref="B311:B311" r:id="Rd272f5bf23c340f7" display="https://etf.dws.com//en-gb/LU0677077884-j-p-morgan-usd-emerging-markets-bond-ucits-etf-2d/"/>
+    <x:hyperlink ref="B312:B312" r:id="Rdeffbe1010e24d12" display="https://etf.dws.com//en-gb/LU0690964092-global-government-bond-ucits-etf-1d-eur-hedged/"/>
+    <x:hyperlink ref="B313:B313" r:id="R5280fdd7360c470d" display="https://etf.dws.com//en-gb/LU0779800910-csi300-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B314:B314" r:id="Ra1df5b666dc64d60" display="https://etf.dws.com//en-gb/LU0838780707-ftse-100-ucits-etf-1c/"/>
+    <x:hyperlink ref="B315:B315" r:id="R90341878a665471d" display="https://etf.dws.com//en-gb/LU0838782315-dax-esg-screened-ucits-etf-1d/"/>
+    <x:hyperlink ref="B316:B316" r:id="R85386721839a466e" display="https://etf.dws.com//en-gb/LU0839027447-nikkei-225-ucits-etf-1d/"/>
+    <x:hyperlink ref="B317:B317" r:id="R9c4e7c107f284bfb" display="https://etf.dws.com//en-gb/LU0846194776-msci-emu-ucits-etf-1d/"/>
+    <x:hyperlink ref="B318:B318" r:id="R848b9af1162745a6" display="https://etf.dws.com//en-gb/LU0875160326-harvest-csi300-ucits-etf-1d/"/>
+    <x:hyperlink ref="B319:B319" r:id="Rc00f01f5d52b4b3a" display="https://etf.dws.com//en-gb/LU0908508731-global-government-bond-ucits-etf-5c/"/>
+    <x:hyperlink ref="B320:B320" r:id="R6840c7f3456b4ef1" display="https://etf.dws.com//en-gb/LU0908508814-global-inflation-linked-bond-ucits-etf-5c/"/>
+    <x:hyperlink ref="B321:B321" r:id="Rf657d630004e4f0b" display="https://etf.dws.com//en-gb/LU0925589839-iboxx-eurozone-government-bond-yield-plus-1-3-ucits-etf-1c/"/>
+    <x:hyperlink ref="B322:B322" r:id="R0bf4ac50e4fa4c53" display="https://etf.dws.com//en-gb/LU0927735406-msci-japan-ucits-etf-2d-usd-hedged/"/>
+    <x:hyperlink ref="B323:B323" r:id="Radc5b6f018fb4753" display="https://etf.dws.com//en-gb/LU0942970103-esg-global-aggregate-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B324:B324" r:id="Rf28b864be2064d7b" display="https://etf.dws.com//en-gb/LU0942970285-esg-global-aggregate-bond-ucits-etf-2c-usd-hedged/"/>
+    <x:hyperlink ref="B325:B325" r:id="R7ad38e13646944bb" display="https://etf.dws.com//en-gb/LU0942970368-esg-global-aggregate-bond-ucits-etf-3d-gbp-hedged/"/>
+    <x:hyperlink ref="B326:B326" r:id="R5d959bc3365144c9" display="https://etf.dws.com//en-gb/LU0942970442-esg-global-aggregate-bond-ucits-etf-4c-chf-hedged/"/>
+    <x:hyperlink ref="B327:B327" r:id="R5cd1945e98f44aa8" display="https://etf.dws.com//en-gb/LU0942970798-esg-global-aggregate-bond-ucits-etf-5c-eur-hedged/"/>
+    <x:hyperlink ref="B328:B328" r:id="R010ad4e2abe74c16" display="https://etf.dws.com//en-gb/LU0943504760-switzerland-ucits-etf-1c/"/>
+    <x:hyperlink ref="B329:B329" r:id="Rf7a2b50c524d4c82" display="https://etf.dws.com//en-gb/LU0952581584-japan-government-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B330:B330" r:id="R2572cc7ae8f1497a" display="https://etf.dws.com//en-gb/LU0962071741-iboxx-eurozone-government-bond-yield-plus-ucits-etf-1d/"/>
+    <x:hyperlink ref="B331:B331" r:id="R1a803e4546e249ce" display="https://etf.dws.com//en-gb/LU0962078753-global-inflation-linked-bond-ucits-etf-1d-eur-hedged/"/>
+    <x:hyperlink ref="B332:B332" r:id="R806ae83147164f71" display="https://etf.dws.com//en-gb/LU0994505336-spain-ucits-etf-1d/"/>
+    <x:hyperlink ref="B333:B333" r:id="R30b3f92489984503" display="https://etf.dws.com//en-gb/LU1094612022-harvest-china-government-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B334:B334" r:id="R2f3b5291d07e414e" display="https://etf.dws.com//en-gb/LU1109939865-rolling-target-maturity-sept-2027-eur-high-yield-ucits-etf-1d/"/>
+    <x:hyperlink ref="B335:B335" r:id="Ree9f2a44e8694a88" display="https://etf.dws.com//en-gb/LU1109941689-rolling-target-maturity-sept-2027-eur-high-yield-ucits-etf-1c/"/>
+    <x:hyperlink ref="B336:B336" r:id="R4a186dfa1c654df5" display="https://etf.dws.com//en-gb/LU1109942653-eur-high-yield-corporate-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B337:B337" r:id="Rea80d6807c4b4624" display="https://etf.dws.com//en-gb/LU1109943388-eur-high-yield-corporate-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B338:B338" r:id="R36365dc365d44ae4" display="https://etf.dws.com//en-gb/LU1127514245-msci-emu-ucits-etf-1c-usd-hedged/"/>
+    <x:hyperlink ref="B339:B339" r:id="Rec677752f8144b6b" display="https://etf.dws.com//en-gb/LU1127516455-msci-emu-ucits-etf-2c-gbp-hedged/"/>
+    <x:hyperlink ref="B340:B340" r:id="Re7a86c01b3964b57" display="https://etf.dws.com//en-gb/LU1184092051-msci-europe-ucits-etf-2c-usd-hedged/"/>
+    <x:hyperlink ref="B341:B341" r:id="R8ab0551eea864e51" display="https://etf.dws.com//en-gb/LU1215827756-msci-japan-ucits-etf-7c-chf-hedged/"/>
+    <x:hyperlink ref="B342:B342" r:id="R161f4e5464a24900" display="https://etf.dws.com//en-gb/LU1215828218-msci-emu-ucits-etf-3c-chf-hedged/"/>
+    <x:hyperlink ref="B343:B343" r:id="Ra41e38b0010546d3" display="https://etf.dws.com//en-gb/LU1221100792-dax-esg-screened-ucits-etf-2c-usd-hedged/"/>
+    <x:hyperlink ref="B344:B344" r:id="Rde327d91e32e404d" display="https://etf.dws.com//en-gb/LU1221102491-dax-esg-screened-ucits-etf-4c-chf-hedged/"/>
+    <x:hyperlink ref="B345:B345" r:id="Rd256017cb2034c46" display="https://etf.dws.com//en-gb/LU1242369327-msci-europe-ucits-etf-1d/"/>
+    <x:hyperlink ref="B346:B346" r:id="R6a88ca1a0fbe4b3a" display="https://etf.dws.com//en-gb/LU1310477036-harvest-csi-a500-ucits-etf-1d/"/>
+    <x:hyperlink ref="B347:B347" r:id="R6c9339e73cf040e1" display="https://etf.dws.com//en-gb/LU1349386927-dax-ucits-etf-1d/"/>
+    <x:hyperlink ref="B348:B348" r:id="R3819bac2cc7a41a6" display="https://etf.dws.com//en-gb/LU1399300455-us-treasuries-ucits-etf-2d-eur-hedged/"/>
+    <x:hyperlink ref="B349:B349" r:id="R20de9b9e8de24d5d" display="https://etf.dws.com//en-gb/LU1772333404-stoxx-europe-600-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B350:B350" r:id="R71e83b6d426042e4" display="https://etf.dws.com//en-gb/LU1875395870-nikkei-225-ucits-etf-2d-eur-hedged/"/>
+    <x:hyperlink ref="B351:B351" r:id="Rfb29b6bf049e4ad8" display="https://etf.dws.com//en-gb/LU1920015440-j-p-morgan-usd-emerging-markets-bond-ucits-etf-2c/"/>
+    <x:hyperlink ref="B352:B352" r:id="Rc35036b97b1342dd" display="https://etf.dws.com//en-gb/LU1920015523-us-treasuries-1-3-ucits-etf-1c/"/>
+    <x:hyperlink ref="B353:B353" r:id="Raaa2ddfdf25e471c" display="https://etf.dws.com//en-gb/LU1920015796-us-treasuries-ucits-etf-1c/"/>
+    <x:hyperlink ref="B354:B354" r:id="R4f326c4ec1c34a44" display="https://etf.dws.com//en-gb/LU2009147591-eurozone-government-bond-ucits-etf-2c-usd-hedged/"/>
+    <x:hyperlink ref="B355:B355" r:id="Rcef7b611b4aa4dc7" display="https://etf.dws.com//en-gb/LU2009147757-s-p-500-swap-ucits-etf-1d/"/>
+    <x:hyperlink ref="B356:B356" r:id="R902b2d3964ff4e3a" display="https://etf.dws.com//en-gb/LU2158769930-j-p-morgan-em-local-government-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B357:B357" r:id="R9005c28fff284bf7" display="https://etf.dws.com//en-gb/LU2178481649-eur-corporate-bond-short-duration-sri-pab-ucits-etf-1c/"/>
+    <x:hyperlink ref="B358:B358" r:id="Rce7da69626ff4abe" display="https://etf.dws.com//en-gb/LU2196470426-nikkei-225-ucits-etf-1c/"/>
+    <x:hyperlink ref="B359:B359" r:id="Re0db9d5f07854b47" display="https://etf.dws.com//en-gb/LU2196472984-s-p-500-swap-ucits-etf-5c-eur-hedged/"/>
+    <x:hyperlink ref="B360:B360" r:id="Rc97fc8444f0441b0" display="https://etf.dws.com//en-gb/LU2196473016-s-p-500-swap-ucits-etf-7c-gbp-hedged/"/>
+    <x:hyperlink ref="B361:B361" r:id="R99fa78022fa447a8" display="https://etf.dws.com//en-gb/LU2263803533-msci-world-swap-ucits-etf-1d/"/>
+    <x:hyperlink ref="B362:B362" r:id="R76a7e2ac122b4e51" display="https://etf.dws.com//en-gb/LU2278080713-bloomberg-commodity-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B363:B363" r:id="Rac06c778109e4c6b" display="https://etf.dws.com//en-gb/LU2296661775-msci-em-asia-screened-swap-ucits-etf-1d/"/>
+    <x:hyperlink ref="B364:B364" r:id="R1451476abbfe4293" display="https://etf.dws.com//en-gb/LU2361257269-j-p-morgan-usd-emerging-markets-bond-ucits-etf-1d-eur-hedged/"/>
+    <x:hyperlink ref="B365:B365" r:id="Rbff0e6115c1a44b3" display="https://etf.dws.com//en-gb/LU2376679564-harvest-msci-china-tech-100-ucits-etf-1c/"/>
+    <x:hyperlink ref="B366:B366" r:id="Rd03ab7ab0cfc4a05" display="https://etf.dws.com//en-gb/LU2385068163-esg-global-government-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B367:B367" r:id="Rcabb8b2d713944ed" display="https://etf.dws.com//en-gb/LU2385068247-esg-global-government-bond-ucits-etf-2d-gbp-hedged/"/>
+    <x:hyperlink ref="B368:B368" r:id="Rb06924f3e91b4f9f" display="https://etf.dws.com//en-gb/LU2385068320-esg-global-government-bond-ucits-etf-3d-usd-hedged/"/>
+    <x:hyperlink ref="B369:B369" r:id="Rdbf4179919c4479f" display="https://etf.dws.com//en-gb/LU2385068593-esg-global-government-bond-ucits-etf-4d-eur-hedged/"/>
+    <x:hyperlink ref="B370:B370" r:id="Rb2d688203e474674" display="https://etf.dws.com//en-gb/LU2456436083-msci-china-ucits-etf-1d/"/>
+    <x:hyperlink ref="B371:B371" r:id="R0c10b3b00a6d4b1c" display="https://etf.dws.com//en-gb/LU2462217071-esg-global-government-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B372:B372" r:id="R563c21c7b4714fa9" display="https://etf.dws.com//en-gb/LU2468423459-esg-eurozone-government-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B373:B373" r:id="Rf6e55627663e4b4e" display="https://etf.dws.com//en-gb/LU2469465822-msci-china-a-screened-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B374:B374" r:id="R33af205db0cb4d7f" display="https://etf.dws.com//en-gb/LU2504532131-tips-us-inflation-linked-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B375:B375" r:id="R1d2917bdb1de486a" display="https://etf.dws.com//en-gb/LU2504532487-eurozone-government-green-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B376:B376" r:id="R5f0896efe7af42ef" display="https://etf.dws.com//en-gb/LU2504537445-eurozone-government-bond-esg-tilted-ucits-etf-1d/"/>
+    <x:hyperlink ref="B377:B377" r:id="R39c39acc7d2d4b07" display="https://etf.dws.com//en-gb/LU2523865728-eurozone-government-bond-7-10-ucits-etf-1d-gbp-hedged/"/>
+    <x:hyperlink ref="B378:B378" r:id="Rd2706ae5afd34b68" display="https://etf.dws.com//en-gb/LU2523865991-eurozone-government-bond-7-10-ucits-etf-2c-usd-hedged/"/>
+    <x:hyperlink ref="B379:B379" r:id="R46fcf99cc2e74126" display="https://etf.dws.com//en-gb/LU2523866023-eurozone-government-bond-ucits-etf-2d-gbp-hedged/"/>
+    <x:hyperlink ref="B380:B380" r:id="R282f7af6e8914542" display="https://etf.dws.com//en-gb/LU2523866296-germany-government-bond-ucits-etf-2d-gbp-hedged/"/>
+    <x:hyperlink ref="B381:B381" r:id="R87a4844a19534bfa" display="https://etf.dws.com//en-gb/LU2523866379-germany-government-bond-ucits-etf-2c-usd-hedged/"/>
+    <x:hyperlink ref="B382:B382" r:id="R407b01ddb8d24bec" display="https://etf.dws.com//en-gb/LU2552296563-iboxx-eurozone-government-bond-yield-plus-1-3-ucits-etf-2d/"/>
+    <x:hyperlink ref="B383:B383" r:id="R9e7d8675df0e4791" display="https://etf.dws.com//en-gb/LU2581375073-msci-usa-swap-ucits-etf-1d/"/>
+    <x:hyperlink ref="B384:B384" r:id="R95a0f3d82c8349b6" display="https://etf.dws.com//en-gb/LU2581375156-stoxx-europe-600-ucits-etf-1d/"/>
+    <x:hyperlink ref="B385:B385" r:id="R872212acde174785" display="https://etf.dws.com//en-gb/LU2581375230-msci-japan-ucits-etf-1d/"/>
+    <x:hyperlink ref="B386:B386" r:id="R337486ec13ab4366" display="https://etf.dws.com//en-gb/LU2606231335-eurozone-government-bond-3-5-ucits-etf-2c-usd-hedged/"/>
+    <x:hyperlink ref="B387:B387" r:id="Rdfc35036cceb4998" display="https://etf.dws.com//en-gb/LU2606231418-eurozone-government-bond-3-5-ucits-etf-2d-gbp-hedged/"/>
+    <x:hyperlink ref="B388:B388" r:id="Ra4588d7b85e04ca0" display="https://etf.dws.com//en-gb/LU2610432036-us-treasuries-ucits-etf-2c-gbp-hedged/"/>
+    <x:hyperlink ref="B389:B389" r:id="R7462715c0e414c2f" display="https://etf.dws.com//en-gb/LU2641054122-eurozone-government-bond-0-1-ucits-etf-1c/"/>
+    <x:hyperlink ref="B390:B390" r:id="Rd1064e196ec14b8b" display="https://etf.dws.com//en-gb/LU2641054551-germany-government-bond-0-1-ucits-etf-1c/"/>
+    <x:hyperlink ref="B391:B391" r:id="R56a06003ac574b13" display="https://etf.dws.com//en-gb/LU2662649412-us-treasuries-10-ucits-etf-1d/"/>
+    <x:hyperlink ref="B392:B392" r:id="R7ad2bfeb45cb41b0" display="https://etf.dws.com//en-gb/LU2662649503-us-treasuries-3-7-ucits-etf-1d/"/>
+    <x:hyperlink ref="B393:B393" r:id="R0f21148320514df5" display="https://etf.dws.com//en-gb/LU2662649685-us-treasuries-7-10-ucits-etf-1d/"/>
+    <x:hyperlink ref="B394:B394" r:id="R0306aa43ae534e77" display="https://etf.dws.com//en-gb/LU2673522830-target-maturity-sept-2027-eur-corporate-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B395:B395" r:id="R762de9ba12c34de8" display="https://etf.dws.com//en-gb/LU2673522913-target-maturity-sept-2029-eur-corporate-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B396:B396" r:id="R546e20966d7d4c27" display="https://etf.dws.com//en-gb/LU2673523051-target-maturity-sept-2033-eur-corporate-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B397:B397" r:id="Rffcd3242180e4b14" display="https://etf.dws.com//en-gb/LU2673523135-target-maturity-sept-2031-eur-corporate-bond-ucits-etf-1c/"/>
+    <x:hyperlink ref="B398:B398" r:id="R002c9c0044954b6e" display="https://etf.dws.com//en-gb/LU2673523218-target-maturity-sept-2027-eur-corporate-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B399:B399" r:id="R1856b3e080a247c8" display="https://etf.dws.com//en-gb/LU2673523309-target-maturity-sept-2029-eur-corporate-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B400:B400" r:id="R7696a55e4402428f" display="https://etf.dws.com//en-gb/LU2673523481-target-maturity-sept-2031-eur-corporate-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B401:B401" r:id="R58b0f7bf196741e7" display="https://etf.dws.com//en-gb/LU2673523564-target-maturity-sept-2033-eur-corporate-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B402:B402" r:id="R5834088c65554c84" display="https://etf.dws.com//en-gb/LU2675291913-msci-emerging-markets-swap-ucits-etf-1d/"/>
+    <x:hyperlink ref="B403:B403" r:id="Rfd44eae2d4f74164" display="https://etf.dws.com//en-gb/LU2755521270-msci-pacific-ex-japan-ucits-etf-1d/"/>
+    <x:hyperlink ref="B404:B404" r:id="R6f1d3dfc92154066" display="https://etf.dws.com//en-gb/LU2788421340-csi500-swap-ucits-etf-1c/"/>
+    <x:hyperlink ref="B405:B405" r:id="R8117a487083c48aa" display="https://etf.dws.com//en-gb/LU2809864296-target-maturity-sept-2030-eur-corporate-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B406:B406" r:id="R24af3b7a66514cbe" display="https://etf.dws.com//en-gb/LU2809864452-target-maturity-sept-2032-eur-corporate-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B407:B407" r:id="Re42183a5a9394518" display="https://etf.dws.com//en-gb/LU2809864619-target-maturity-sept-2034-eur-corporate-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B408:B408" r:id="Rd53e23a18b474e1d" display="https://etf.dws.com//en-gb/LU2810185665-target-maturity-sept-2028-eur-corporate-bond-ucits-etf-1d/"/>
+    <x:hyperlink ref="B409:B409" r:id="R45656e5b11c0408c" display="https://etf.dws.com//en-gb/LU2859297330-world-small-cap-green-tech-innovators-ucits-etf-1c/"/>
+    <x:hyperlink ref="B410:B410" r:id="Rb685445e071b4788" display="https://etf.dws.com//en-gb/LU2859392081-world-green-tech-innovators-ucits-etf-1c/"/>
+    <x:hyperlink ref="B411:B411" r:id="Rfe76f46c7b0b4c54" display="https://etf.dws.com//en-gb/LU2903252349-scalable-msci-ac-world-xtrackers-ucits-etf-1c/"/>
+    <x:hyperlink ref="B412:B412" r:id="R8a59bae6c6e24fec" display="https://etf.dws.com//en-gb/LU2928641757-msci-taiwan-ucits-etf-1d/"/>
+    <x:hyperlink ref="B413:B413" r:id="R53c551243fa64a23" display="https://etf.dws.com//en-gb/LU3003217554-eurozone-government-bond-1-3-ucits-etf-2c-usd-hedged/"/>
+    <x:hyperlink ref="B414:B414" r:id="R5a94049c905b45bb" display="https://etf.dws.com//en-gb/LU3003217638-eurozone-government-bond-1-3-ucits-etf-2d-gbp-hedged/"/>
+    <x:hyperlink ref="B415:B415" r:id="R80377fbbcdd74376" display="https://etf.dws.com//en-gb/LU3003217711-eurozone-government-bond-5-7-ucits-etf-2c-usd-hedged/"/>
+    <x:hyperlink ref="B416:B416" r:id="Ree6d448606c54aa2" display="https://etf.dws.com//en-gb/LU3003217984-eurozone-government-bond-5-7-ucits-etf-1d-gbp-hedged/"/>
+    <x:hyperlink ref="B417:B417" r:id="R9d5953c2bb7d4fe6" display="https://etf.dws.com//en-gb/LU3003218016-australia-government-bond-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B418:B418" r:id="R94820648b1b746c4" display="https://etf.dws.com//en-gb/LU3003218107-australia-government-bond-ucits-etf-3c-usd-hedged/"/>
+    <x:hyperlink ref="B419:B419" r:id="R2fe09319d5b64f6f" display="https://etf.dws.com//en-gb/LU3003218362-australia-government-bond-ucits-etf-1d-gbp-hedged/"/>
+    <x:hyperlink ref="B420:B420" r:id="R3fdfb6d741884127" display="https://etf.dws.com//en-gb/LU3003218446-japan-government-bond-ucits-etf-2c-eur-hedged/"/>
+    <x:hyperlink ref="B421:B421" r:id="Re416375bedb34cc4" display="https://etf.dws.com//en-gb/LU3003218792-japan-government-bond-ucits-etf-3c-usd-hedged/"/>
+    <x:hyperlink ref="B422:B422" r:id="R73f314b85a1c4f61" display="https://etf.dws.com//en-gb/LU3003218958-japan-government-bond-ucits-etf-2d-gbp-hedged/"/>
+    <x:hyperlink ref="B423:B423" r:id="R879b16edb4be4b4e" display="https://etf.dws.com//en-gb/LU3061478973-europe-defence-technologies-ucits-etf-1c/"/>
+    <x:hyperlink ref="B424:B424" r:id="Redb885d5859f4469" display="https://etf.dws.com//en-gb/LU3116008346-diversified-portfolio-20-equity-ucits-etf-1c/"/>
+    <x:hyperlink ref="B425:B425" r:id="Rf593d64f3c8b4644" display="https://etf.dws.com//en-gb/LU3116008429-diversified-portfolio-40-equity-ucits-etf-1c/"/>
+    <x:hyperlink ref="B426:B426" r:id="R0ff7cf98f43949fe" display="https://etf.dws.com//en-gb/LU3116008692-diversified-portfolio-60-equity-ucits-etf-1c/"/>
+    <x:hyperlink ref="B427:B427" r:id="R491325f88daf43e4" display="https://etf.dws.com//en-gb/LU3116008775-diversified-portfolio-80-equity-ucits-etf-1c/"/>
+    <x:hyperlink ref="B428:B428" r:id="R034bd14e665945c0" display="https://etf.dws.com//en-gb/LU3121019551-global-government-bond-ucits-etf-3d-chf-hedged/"/>
+    <x:hyperlink ref="B429:B429" r:id="Rc04208c5c4e447d6" display="https://etf.dws.com//en-gb/LU3123443510-salam-usd-global-aggregate-sukuk-ucits-etf-1d/"/>
+    <x:hyperlink ref="B430:B430" r:id="Red8f89700c024560" display="https://etf.dws.com//en-gb/LU3184977026-msci-world-swap-ucits-etf-ic-gbp-unlisted/"/>
+    <x:hyperlink ref="B431:B431" r:id="R3520dab09b0847ec" display="https://etf.dws.com//en-gb/LU3184977299-msci-europe-ucits-etf-ic-eur-unlisted/"/>
+    <x:hyperlink ref="B432:B432" r:id="R2c7de443492041d7" display="https://etf.dws.com//en-gb/LU3184977372-msci-usa-swap-ucits-etf-ic-gbp-unlisted/"/>
+    <x:hyperlink ref="B433:B433" r:id="R2622f925e20a44e6" display="https://etf.dws.com//en-gb/LU3184977455-msci-emerging-markets-swap-ucits-etf-ic-gbp-unlisted/"/>
+    <x:hyperlink ref="B434:B434" r:id="R02a582c54793451b" display="https://etf.dws.com//en-gb/LU3184977612-s-p-500-swap-ucits-etf-ic-gbp-unlisted/"/>
+    <x:hyperlink ref="B435:B435" r:id="R671bba88e9294368" display="https://etf.dws.com//en-gb/LU3184977703-ftse-100-ucits-etf-ic-gbp-unlisted/"/>
+    <x:hyperlink ref="B436:B436" r:id="R2f322fea0f6642f5" display="https://etf.dws.com//en-gb/LU3198621024-s-p-500-swap-ucits-etf-ic-usd-unlisted/"/>
+    <x:hyperlink ref="B437:B437" r:id="R11a4703930b94916" display="https://etf.dws.com//en-gb/LU3284391318-global-government-bond-ucits-etf-4d/"/>
+    <x:hyperlink ref="B438:B438" r:id="R962ace8710e041f5" display="https://etf.dws.com//en-gb/LU3313127113-eurozone-government-bond-ucits-etf-ic-eur-unlisted/"/>
+    <x:hyperlink ref="B439:B439" r:id="Re0ac575575bb49e3" display="https://etf.dws.com//en-gb/LU3353962601-msci-world-swap-ucits-etf-ic-eur-unlisted/"/>
+    <x:hyperlink ref="B440:B440" r:id="R148e9d6233e44f31" display="https://etf.dws.com//en-gb/LU3353962783-s-p-500-swap-ucits-etf-ic-eur-unlisted/"/>
+    <x:hyperlink ref="B441:B441" r:id="R0109a374a6e3425f" display="https://etf.dws.com//en-gb/LU3353962866-stoxx-global-select-dividend-100-swap-ucits-etf-ic-usd-unlisted/"/>
+    <x:hyperlink ref="B442:B442" r:id="R821f1744f8954f2f" display="https://etf.dws.com//en-gb/LU3353962940-stoxx-europe-600-ucits-etf-ic-eur-unlisted/"/>
+    <x:hyperlink ref="B443:B443" r:id="R84da83451f734fc8" display="https://etf.dws.com//en-gb/LU3370249040-bloomberg-commodity-swap-ucits-etf-3c-gbp-hedged/"/>
+    <x:hyperlink ref="B444:B444" r:id="R0e767be10a5449b0" display="https://etf.dws.com//en-gb/LU3375213041-msci-world-swap-ucits-etf-ic-usd-unlisted/"/>
   </x:hyperlinks>
   <x:pageMargins left="0.17" right="0.17" top="0.17" bottom="0.17" header="0" footer="0.3"/>
   <x:pageSetup orientation="landscape"/>
   <x:drawing r:id="rId2"/>
   <x:tableParts count="1">
-    <x:tablePart r:id="R90dae02d21e949ae"/>
+    <x:tablePart r:id="R4c3a7fe85f2c4205"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>